<commit_message>
docs(control): update dashboard through Phase 21, fix route count
Roadmap/Todo/Modules/API Endpoints sheets updated for Trust & Safety
(21 routes, 131 total endpoints, 25 commits). Also fixes a miscount in
trustsafety/README.md (said 18 routes, actually 21).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D111" headerRowCount="1">
-  <autoFilter ref="A1:D111"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D114" headerRowCount="1">
+  <autoFilter ref="A1:D114"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -252,8 +252,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F24" headerRowCount="1">
-  <autoFilter ref="A1:F24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F25" headerRowCount="1">
+  <autoFilter ref="A1:F25"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="Service"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E111" headerRowCount="1">
-  <autoFilter ref="A1:E111"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E132" headerRowCount="1">
+  <autoFilter ref="A1:E132"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Method"/>
     <tableColumn id="2" name="Path"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>20 / 30</t>
+          <t>21 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>70%</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>131</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0018</t>
+          <t>data/migrations/0001-0019</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1371,9 +1371,9 @@
       <c r="A22" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Reusable Block/Mute/Report/ModerationCase/Suspension/Ban/Appeal, plus rate limiting, spam protection, abuse signals. Product-specific report reasons pluggable.</t>
+          <t>Mute/Report-&gt;ModerationCase (deduplicated)/Suspension/Ban/Appeal - Block reuses Phase 8's relationships, not duplicated. A new requireActive middleware makes Suspension/Ban actually restrict access platform-wide from one place. New shared ratelimit package (Valkey-backed) gates report spam; a critical AbuseSignal auto-opens a case.</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7af4c58</t>
         </is>
       </c>
     </row>
@@ -1396,9 +1396,9 @@
       <c r="A23" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D111"/>
+  <dimension ref="A1:D114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
@@ -1993,14 +1993,14 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 21: Trust &amp; Safety implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
@@ -2009,18 +2009,14 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -2029,32 +2025,32 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2065,12 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2089,30 +2085,34 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr"/>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr"/>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr"/>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
@@ -2198,21 +2198,17 @@
       <c r="A34" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -2225,18 +2221,18 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
@@ -2245,39 +2241,47 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr"/>
+          <t>Privacy: relationships/groups/messaging as participants</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B38" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
@@ -2286,14 +2290,14 @@
       <c r="A39" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: ModerationCase</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
@@ -2302,9 +2306,9 @@
       <c r="A40" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
@@ -2318,9 +2322,9 @@
       <c r="A41" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B41" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
@@ -2334,14 +2338,14 @@
       <c r="A42" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
@@ -2350,14 +2354,14 @@
       <c r="A43" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B43" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
@@ -2366,14 +2370,14 @@
       <c r="A44" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B44" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2382,14 +2386,14 @@
       <c r="A45" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B45" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2398,37 +2402,37 @@
       <c r="A46" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B46" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B47" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>21</v>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Payment model</t>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
@@ -2437,14 +2441,18 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Entitlement model (kept separate from Payment)</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B49" s="13" t="inlineStr">
         <is>
@@ -2453,10 +2461,14 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: provider abstraction (implement first)</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
@@ -2469,7 +2481,7 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Stripe adapter</t>
+          <t>Billing / Entitlements: Payment model</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
@@ -2485,7 +2497,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Apple IAP adapter</t>
+          <t>Billing / Entitlements: Entitlement model (kept separate from Payment)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr"/>
@@ -2501,14 +2513,14 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Google Play adapter</t>
+          <t>Billing / Entitlements: provider abstraction (implement first)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B53" s="13" t="inlineStr">
         <is>
@@ -2517,14 +2529,14 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
+          <t>Billing / Entitlements: Stripe adapter</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B54" s="13" t="inlineStr">
         <is>
@@ -2533,14 +2545,14 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path</t>
+          <t>Billing / Entitlements: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B55" s="13" t="inlineStr">
         <is>
@@ -2549,14 +2561,14 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake</t>
+          <t>Billing / Entitlements: Google Play adapter</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
@@ -2565,14 +2577,14 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
+          <t>Analytics: generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B57" s="13" t="inlineStr">
         <is>
@@ -2581,14 +2593,14 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing</t>
+          <t>Analytics: keep operational DBs out of the analytics path</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B58" s="13" t="inlineStr">
         <is>
@@ -2597,7 +2609,7 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas</t>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr"/>
@@ -2613,7 +2625,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
@@ -2629,7 +2641,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking</t>
+          <t>AI Gateway: model routing</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
@@ -2645,7 +2657,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration</t>
+          <t>AI Gateway: quotas</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
@@ -2661,7 +2673,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
@@ -2677,7 +2689,7 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts</t>
+          <t>AI Gateway: cost tracking</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
@@ -2693,14 +2705,14 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback</t>
+          <t>AI Gateway: audit integration</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B65" s="13" t="inlineStr">
         <is>
@@ -2709,14 +2721,14 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: control-plane UI in apps/admin</t>
+          <t>AI Gateway: prompt/version metadata</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B66" s="13" t="inlineStr">
         <is>
@@ -2725,14 +2737,14 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Applications</t>
+          <t>AI Gateway: timeouts</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B67" s="13" t="inlineStr">
         <is>
@@ -2741,7 +2753,7 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
+          <t>AI Gateway: fallback</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr"/>
@@ -2757,7 +2769,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Roles/Permissions</t>
+          <t>Admin Portal: control-plane UI in apps/admin</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
@@ -2773,7 +2785,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Tenants/Relationships</t>
+          <t>Admin Portal: visibility: Applications</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
@@ -2789,7 +2801,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Messages/Notifications</t>
+          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
@@ -2805,7 +2817,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Files/Jobs</t>
+          <t>Admin Portal: visibility: Roles/Permissions</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
@@ -2821,7 +2833,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Feature flags/Configuration</t>
+          <t>Admin Portal: visibility: Tenants/Relationships</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
@@ -2837,7 +2849,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Moderation/Audit</t>
+          <t>Admin Portal: visibility: Messages/Notifications</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2853,7 +2865,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: System health/Deployments</t>
+          <t>Admin Portal: visibility: Files/Jobs</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2869,14 +2881,14 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
+          <t>Admin Portal: visibility: Feature flags/Configuration</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
@@ -2885,14 +2897,14 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: visibility: Moderation/Audit</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
@@ -2901,14 +2913,14 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
+          <t>Admin Portal: visibility: System health/Deployments</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B78" s="13" t="inlineStr">
         <is>
@@ -2917,7 +2929,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
+          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
@@ -2933,14 +2945,14 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
@@ -2949,14 +2961,14 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
+          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
@@ -2965,14 +2977,14 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
+          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
@@ -2981,7 +2993,7 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
+          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
@@ -2997,7 +3009,7 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
+          <t>SDKs: Flutter SDK</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
@@ -3013,7 +3025,7 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
@@ -3029,7 +3041,7 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
@@ -3045,7 +3057,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr"/>
@@ -3061,14 +3073,14 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
@@ -3077,14 +3089,14 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
@@ -3093,14 +3105,14 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
@@ -3109,7 +3121,7 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr"/>
@@ -3125,7 +3137,7 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr"/>
@@ -3141,7 +3153,7 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr"/>
@@ -3157,7 +3169,7 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr"/>
@@ -3173,7 +3185,7 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr"/>
@@ -3189,7 +3201,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr"/>
@@ -3205,7 +3217,7 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr"/>
@@ -3221,7 +3233,7 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr"/>
@@ -3237,7 +3249,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr"/>
@@ -3253,7 +3265,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr"/>
@@ -3269,7 +3281,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr"/>
@@ -3285,14 +3297,14 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
@@ -3301,14 +3313,14 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
@@ -3317,14 +3329,14 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
@@ -3333,7 +3345,7 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr"/>
@@ -3349,14 +3361,14 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
@@ -3365,14 +3377,14 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
@@ -3381,14 +3393,14 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
@@ -3397,7 +3409,7 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr"/>
@@ -3413,7 +3425,7 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>AI Development Context: every module: README</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
@@ -3429,7 +3441,7 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>AI Development Context: every module: ownership metadata</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
@@ -3445,10 +3457,58 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
+          <t>AI Development Context: every module: dependencies</t>
+        </is>
+      </c>
+      <c r="D111" s="11" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B112" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B113" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D113" s="11" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B114" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C114" s="11" t="inlineStr">
+        <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D111" s="11" t="inlineStr"/>
+      <c r="D114" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3464,7 +3524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4240,6 +4300,38 @@
       <c r="F24" s="11" t="inlineStr">
         <is>
           <t>Phase 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Mute/Report/ModerationCase/Suspension/Ban/Appeal/AbuseSignal - Block reuses Phase 8's relationships</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>mutes, moderation_cases, reports, suspensions, bans, appeals, abuse_signals</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Self for own mutes/appeals; moderator-or-admin for case/suspension/ban management</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Phase 21</t>
         </is>
       </c>
     </row>
@@ -4257,7 +4349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E111"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -6981,6 +7073,545 @@
       <c r="E111" s="11" t="inlineStr">
         <is>
           <t>a self-deleted user must use an admin to check this</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/mutes</t>
+        </is>
+      </c>
+      <c r="C112" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D112" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self)</t>
+        </is>
+      </c>
+      <c r="E112" s="11" t="inlineStr">
+        <is>
+          <t>one-directional, silent</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/mutes</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D113" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self)</t>
+        </is>
+      </c>
+      <c r="E113" s="11" t="inlineStr">
+        <is>
+          <t>exempt from requireActive - always reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="11" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/mutes/{userId}</t>
+        </is>
+      </c>
+      <c r="C114" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self)</t>
+        </is>
+      </c>
+      <c r="E114" s="11" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/reports</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D115" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self)</t>
+        </is>
+      </c>
+      <c r="E115" s="11" t="inlineStr">
+        <is>
+          <t>rate-limited 5/hour; dedupes onto one case</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/reports/{id}</t>
+        </is>
+      </c>
+      <c r="C116" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D116" s="11" t="inlineStr">
+        <is>
+          <t>Reporter or moderator/admin</t>
+        </is>
+      </c>
+      <c r="E116" s="11" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/cases</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D117" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E117" s="11" t="inlineStr">
+        <is>
+          <t>?status=</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/cases/{id}</t>
+        </is>
+      </c>
+      <c r="C118" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D118" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E118" s="11" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/cases/{id}/reports</t>
+        </is>
+      </c>
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D119" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E119" s="11" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="11" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/cases/{id}/assign</t>
+        </is>
+      </c>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D120" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E120" s="11" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="11" t="inlineStr">
+        <is>
+          <t>PATCH</t>
+        </is>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/cases/{id}</t>
+        </is>
+      </c>
+      <c r="C121" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D121" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E121" s="11" t="inlineStr">
+        <is>
+          <t>resolve/dismiss</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/suspensions</t>
+        </is>
+      </c>
+      <c r="C122" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D122" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E122" s="11" t="inlineStr">
+        <is>
+          <t>temporary, EndsAt required</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/suspensions</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D123" s="11" t="inlineStr">
+        <is>
+          <t>Self or moderator/admin</t>
+        </is>
+      </c>
+      <c r="E123" s="11" t="inlineStr">
+        <is>
+          <t>?userId=</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/suspensions/{id}/lift</t>
+        </is>
+      </c>
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D124" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E124" s="11" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/bans</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D125" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E125" s="11" t="inlineStr">
+        <is>
+          <t>permanent until lifted</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/bans</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>Self or moderator/admin</t>
+        </is>
+      </c>
+      <c r="E126" s="11" t="inlineStr">
+        <is>
+          <t>?userId=</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/bans/{id}/lift</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D127" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E127" s="11" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/appeals</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self, must own target)</t>
+        </is>
+      </c>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>exempt from requireActive - always reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/appeals</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D129" s="11" t="inlineStr">
+        <is>
+          <t>Self or moderator/admin</t>
+        </is>
+      </c>
+      <c r="E129" s="11" t="inlineStr">
+        <is>
+          <t>exempt from requireActive - always reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/appeals/{id}/review</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E130" s="11" t="inlineStr">
+        <is>
+          <t>approving lifts the target restriction</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/signals</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D131" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated</t>
+        </is>
+      </c>
+      <c r="E131" s="11" t="inlineStr">
+        <is>
+          <t>critical severity auto-opens a case</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>/v1/trustsafety/signals</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>trustsafety</t>
+        </is>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>Moderator or platform.admin</t>
+        </is>
+      </c>
+      <c r="E132" s="11" t="inlineStr">
+        <is>
+          <t>?resourceType=&amp;resourceId=</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 22
Roadmap/Todo/Modules/API Endpoints sheets updated for Billing /
Entitlements (6 routes, 137 total endpoints, 28 commits, 46/114 todo
items done).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D114" headerRowCount="1">
-  <autoFilter ref="A1:D114"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D115" headerRowCount="1">
+  <autoFilter ref="A1:D115"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -252,8 +252,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F25" headerRowCount="1">
-  <autoFilter ref="A1:F25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F27" headerRowCount="1">
+  <autoFilter ref="A1:F27"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="Service"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E132" headerRowCount="1">
-  <autoFilter ref="A1:E132"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E138" headerRowCount="1">
+  <autoFilter ref="A1:E138"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Method"/>
     <tableColumn id="2" name="Path"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>21 / 30</t>
+          <t>22 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>70%</t>
+          <t>73%</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>137</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0019</t>
+          <t>data/migrations/0001-0020</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1396,9 +1396,9 @@
       <c r="A23" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -1408,12 +1408,12 @@
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>Separate Payment from Entitlement - products ask 'has entitlement X', never 'is the Stripe subscription active'. Provider abstraction first (Stripe, Apple IAP, Google Play).</t>
+          <t>Entitlement (platform truth, HasEntitlement) kept separate from Payment (provider transaction record). PaymentProvider abstraction + registry; billing/stripe implements Stripe's real webhook HMAC signature scheme, live-validated without a Stripe account via self-signed test payloads. Apple IAP/Google Play deliberately deferred - no sandbox credentials available.</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8fcc87f</t>
         </is>
       </c>
     </row>
@@ -1421,9 +1421,9 @@
       <c r="A24" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D114"/>
+  <dimension ref="A1:D115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2000,7 +2000,7 @@
     </row>
     <row r="23">
       <c r="A23" s="9" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
@@ -2009,14 +2009,14 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 22: Billing / Entitlements implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -2025,18 +2025,14 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -2045,32 +2041,32 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2081,12 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2105,30 +2101,34 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr"/>
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr"/>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
@@ -2214,21 +2214,17 @@
       <c r="A35" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
@@ -2241,32 +2237,32 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2281,10 +2277,14 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D38" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr"/>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2434,21 +2434,17 @@
       <c r="A48" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B48" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
@@ -2461,18 +2457,18 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
@@ -2481,23 +2477,27 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Payment model</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Entitlement model (kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr"/>
@@ -2506,14 +2506,14 @@
       <c r="A52" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: provider abstraction (implement first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
@@ -2522,14 +2522,14 @@
       <c r="A53" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Stripe adapter</t>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
@@ -2538,17 +2538,21 @@
       <c r="A54" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Apple IAP adapter</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="inlineStr"/>
+          <t>Billing: Stripe adapter</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -2561,14 +2565,18 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Billing / Entitlements: Google Play adapter</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="inlineStr"/>
+          <t>Billing: Apple IAP adapter</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B56" s="13" t="inlineStr">
         <is>
@@ -2577,10 +2585,14 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
@@ -2593,7 +2605,7 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path</t>
+          <t>Analytics: generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr"/>
@@ -2609,14 +2621,14 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake</t>
+          <t>Analytics: keep operational DBs out of the analytics path</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B59" s="13" t="inlineStr">
         <is>
@@ -2625,7 +2637,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
@@ -2641,7 +2653,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing</t>
+          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
@@ -2657,7 +2669,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas</t>
+          <t>AI Gateway: model routing</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
@@ -2673,7 +2685,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: quotas</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
@@ -2689,7 +2701,7 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
@@ -2705,7 +2717,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration</t>
+          <t>AI Gateway: cost tracking</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
@@ -2721,7 +2733,7 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata</t>
+          <t>AI Gateway: audit integration</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr"/>
@@ -2737,7 +2749,7 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts</t>
+          <t>AI Gateway: prompt/version metadata</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr"/>
@@ -2753,14 +2765,14 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback</t>
+          <t>AI Gateway: timeouts</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B68" s="13" t="inlineStr">
         <is>
@@ -2769,7 +2781,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: control-plane UI in apps/admin</t>
+          <t>AI Gateway: fallback</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
@@ -2785,7 +2797,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Applications</t>
+          <t>Admin Portal: control-plane UI in apps/admin</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
@@ -2801,7 +2813,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
+          <t>Admin Portal: visibility: Applications</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
@@ -2817,7 +2829,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Roles/Permissions</t>
+          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
@@ -2833,7 +2845,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Tenants/Relationships</t>
+          <t>Admin Portal: visibility: Roles/Permissions</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
@@ -2849,7 +2861,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Messages/Notifications</t>
+          <t>Admin Portal: visibility: Tenants/Relationships</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2865,7 +2877,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Files/Jobs</t>
+          <t>Admin Portal: visibility: Messages/Notifications</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2881,7 +2893,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Feature flags/Configuration</t>
+          <t>Admin Portal: visibility: Files/Jobs</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
@@ -2897,7 +2909,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Moderation/Audit</t>
+          <t>Admin Portal: visibility: Feature flags/Configuration</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
@@ -2913,7 +2925,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: System health/Deployments</t>
+          <t>Admin Portal: visibility: Moderation/Audit</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
@@ -2929,14 +2941,14 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
+          <t>Admin Portal: visibility: System health/Deployments</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B79" s="13" t="inlineStr">
         <is>
@@ -2945,7 +2957,7 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr"/>
@@ -2961,7 +2973,7 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
@@ -2977,7 +2989,7 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
+          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
@@ -2993,14 +3005,14 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
+          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
@@ -3009,7 +3021,7 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
+          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
@@ -3025,7 +3037,7 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
+          <t>SDKs: Flutter SDK</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
@@ -3041,7 +3053,7 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
@@ -3057,7 +3069,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr"/>
@@ -3073,7 +3085,7 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr"/>
@@ -3089,7 +3101,7 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr"/>
@@ -3105,7 +3117,7 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr"/>
@@ -3121,14 +3133,14 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
@@ -3137,7 +3149,7 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr"/>
@@ -3153,7 +3165,7 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr"/>
@@ -3169,7 +3181,7 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr"/>
@@ -3185,7 +3197,7 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr"/>
@@ -3201,7 +3213,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr"/>
@@ -3217,7 +3229,7 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr"/>
@@ -3233,7 +3245,7 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr"/>
@@ -3249,7 +3261,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr"/>
@@ -3265,7 +3277,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr"/>
@@ -3281,7 +3293,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr"/>
@@ -3297,7 +3309,7 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr"/>
@@ -3313,7 +3325,7 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr"/>
@@ -3329,7 +3341,7 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr"/>
@@ -3345,14 +3357,14 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
@@ -3361,7 +3373,7 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr"/>
@@ -3377,7 +3389,7 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr"/>
@@ -3393,7 +3405,7 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr"/>
@@ -3409,14 +3421,14 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
@@ -3425,7 +3437,7 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
@@ -3441,7 +3453,7 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>AI Development Context: every module: README</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
@@ -3457,7 +3469,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>AI Development Context: every module: ownership metadata</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr"/>
@@ -3473,7 +3485,7 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>AI Development Context: every module: dependencies</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr"/>
@@ -3489,7 +3501,7 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>AI Development Context: every module: API contract</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr"/>
@@ -3505,10 +3517,26 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D114" s="11" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B115" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D114" s="11" t="inlineStr"/>
+      <c r="D115" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3524,7 +3552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4332,6 +4360,70 @@
       <c r="F25" s="11" t="inlineStr">
         <is>
           <t>Phase 21</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Entitlement (platform truth) kept separate from Payment (provider transaction record); PaymentProvider abstraction + registry</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>entitlements, payments</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>Self for own entitlements/payments; platform.admin for manual grants</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Phase 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>billing/stripe</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Real Stripe webhook HMAC-SHA256 signature verification - the one live-testable PaymentProvider this phase ships</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>none (stateless verification)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>n/a (provider-signature-authenticated, not a Bearer route)</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Phase 22</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E132"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7612,6 +7704,164 @@
       <c r="E132" s="11" t="inlineStr">
         <is>
           <t>?resourceType=&amp;resourceId=</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/entitlements</t>
+        </is>
+      </c>
+      <c r="C133" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D133" s="11" t="inlineStr">
+        <is>
+          <t>Self or platform.admin</t>
+        </is>
+      </c>
+      <c r="E133" s="11" t="inlineStr">
+        <is>
+          <t>?userId=</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B134" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/entitlements/check/{key}</t>
+        </is>
+      </c>
+      <c r="C134" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (self)</t>
+        </is>
+      </c>
+      <c r="E134" s="11" t="inlineStr">
+        <is>
+          <t>the literal 'do I have entitlement X' check</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B135" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/entitlements</t>
+        </is>
+      </c>
+      <c r="C135" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D135" s="11" t="inlineStr">
+        <is>
+          <t>platform.admin</t>
+        </is>
+      </c>
+      <c r="E135" s="11" t="inlineStr">
+        <is>
+          <t>manual grant; source always "manual:&lt;adminId&gt;"</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B136" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/entitlements/{id}/revoke</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D136" s="11" t="inlineStr">
+        <is>
+          <t>platform.admin</t>
+        </is>
+      </c>
+      <c r="E136" s="11" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/payments</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr">
+        <is>
+          <t>Self or platform.admin</t>
+        </is>
+      </c>
+      <c r="E137" s="11" t="inlineStr">
+        <is>
+          <t>?userId=</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>/v1/billing/webhooks/{provider}</t>
+        </is>
+      </c>
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>billing</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>Provider webhook signature (no Bearer token)</t>
+        </is>
+      </c>
+      <c r="E138" s="11" t="inlineStr">
+        <is>
+          <t>the one route on this platform with no requireUser/requireActive</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 23
Roadmap/Todo/Modules/API Endpoints sheets updated for Analytics (2
routes, 139 total endpoints, 30 commits, 50/116 todo items done).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D115" headerRowCount="1">
-  <autoFilter ref="A1:D115"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D117" headerRowCount="1">
+  <autoFilter ref="A1:D117"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -252,8 +252,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F27" headerRowCount="1">
-  <autoFilter ref="A1:F27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F29" headerRowCount="1">
+  <autoFilter ref="A1:F29"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="Service"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E138" headerRowCount="1">
-  <autoFilter ref="A1:E138"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E140" headerRowCount="1">
+  <autoFilter ref="A1:E140"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Method"/>
     <tableColumn id="2" name="Path"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>22 / 30</t>
+          <t>23 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>77%</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>139</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>21</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0020</t>
+          <t>data/migrations/0001-0021</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1421,9 +1421,9 @@
       <c r="A24" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context). Operational DBs must not become analytics DBs - pipeline foundation for ClickHouse/warehouse/data lake.</t>
+          <t>Generic event envelope, matching the roadmap's own field names verbatim. analytics_events is a landing buffer, never queried for analytics - a new worker pipeline batches unflushed rows as NDJSON into MinIO/S3 (a real data-lake landing pattern). Track is this platform's one open, unauthenticated write endpoint, IP-rate-limited instead of Bearer-gated.</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>aa207ae</t>
         </is>
       </c>
     </row>
@@ -1446,9 +1446,9 @@
       <c r="A25" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D115"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2016,7 +2016,7 @@
     </row>
     <row r="24">
       <c r="A24" s="9" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
@@ -2025,14 +2025,14 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 23: Analytics implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -2041,18 +2041,14 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
@@ -2061,32 +2057,32 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2101,12 +2097,12 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2121,30 +2117,34 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr"/>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
@@ -2230,21 +2230,17 @@
       <c r="A36" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
@@ -2257,32 +2253,32 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2297,10 +2293,14 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr"/>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
@@ -2450,21 +2450,17 @@
       <c r="A49" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D49" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="9" t="n">
@@ -2477,30 +2473,34 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B51" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>21</v>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Billing: Payment model (provider-specific transaction record)</t>
-        </is>
-      </c>
-      <c r="D51" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
@@ -2545,32 +2545,28 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Billing: Stripe adapter</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="inlineStr">
-        <is>
-          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
-        </is>
-      </c>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Billing: Apple IAP adapter</t>
+          <t>Billing: Stripe adapter</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
         </is>
       </c>
     </row>
@@ -2585,18 +2581,18 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Billing: Google Play adapter</t>
+          <t>Billing: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B57" s="13" t="inlineStr">
         <is>
@@ -2605,23 +2601,27 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic analytics event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path</t>
+          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr"/>
@@ -2630,37 +2630,37 @@
       <c r="A59" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake</t>
+          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>23</v>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B61" s="13" t="inlineStr">
         <is>
@@ -2669,10 +2669,14 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="inlineStr"/>
+          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
@@ -2685,7 +2689,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas</t>
+          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
@@ -2701,7 +2705,7 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: model routing</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
@@ -2717,7 +2721,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking</t>
+          <t>AI Gateway: quotas</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
@@ -2733,7 +2737,7 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr"/>
@@ -2749,7 +2753,7 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata</t>
+          <t>AI Gateway: cost tracking</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr"/>
@@ -2765,7 +2769,7 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts</t>
+          <t>AI Gateway: audit integration</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr"/>
@@ -2781,14 +2785,14 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback</t>
+          <t>AI Gateway: prompt/version metadata</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B69" s="13" t="inlineStr">
         <is>
@@ -2797,14 +2801,14 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: control-plane UI in apps/admin</t>
+          <t>AI Gateway: timeouts</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B70" s="13" t="inlineStr">
         <is>
@@ -2813,7 +2817,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Applications</t>
+          <t>AI Gateway: fallback</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
@@ -2829,7 +2833,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
+          <t>Admin Portal: control-plane UI in apps/admin</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
@@ -2845,7 +2849,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Roles/Permissions</t>
+          <t>Admin Portal: visibility: Applications</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
@@ -2861,7 +2865,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Tenants/Relationships</t>
+          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2877,7 +2881,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Messages/Notifications</t>
+          <t>Admin Portal: visibility: Roles/Permissions</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2893,7 +2897,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Files/Jobs</t>
+          <t>Admin Portal: visibility: Tenants/Relationships</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
@@ -2909,7 +2913,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Feature flags/Configuration</t>
+          <t>Admin Portal: visibility: Messages/Notifications</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
@@ -2925,7 +2929,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Moderation/Audit</t>
+          <t>Admin Portal: visibility: Files/Jobs</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
@@ -2941,7 +2945,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: System health/Deployments</t>
+          <t>Admin Portal: visibility: Feature flags/Configuration</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
@@ -2957,14 +2961,14 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
+          <t>Admin Portal: visibility: Moderation/Audit</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B80" s="13" t="inlineStr">
         <is>
@@ -2973,14 +2977,14 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: visibility: System health/Deployments</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B81" s="13" t="inlineStr">
         <is>
@@ -2989,7 +2993,7 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
+          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
@@ -3005,7 +3009,7 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
@@ -3021,14 +3025,14 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
+          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
@@ -3037,14 +3041,14 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
+          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
@@ -3053,7 +3057,7 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
+          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
@@ -3069,7 +3073,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
+          <t>SDKs: Flutter SDK</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr"/>
@@ -3085,7 +3089,7 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr"/>
@@ -3101,7 +3105,7 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr"/>
@@ -3117,7 +3121,7 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr"/>
@@ -3133,7 +3137,7 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr"/>
@@ -3149,14 +3153,14 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B92" s="13" t="inlineStr">
         <is>
@@ -3165,14 +3169,14 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B93" s="13" t="inlineStr">
         <is>
@@ -3181,7 +3185,7 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr"/>
@@ -3197,7 +3201,7 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr"/>
@@ -3213,7 +3217,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr"/>
@@ -3229,7 +3233,7 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr"/>
@@ -3245,7 +3249,7 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr"/>
@@ -3261,7 +3265,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr"/>
@@ -3277,7 +3281,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr"/>
@@ -3293,7 +3297,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr"/>
@@ -3309,7 +3313,7 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr"/>
@@ -3325,7 +3329,7 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr"/>
@@ -3341,7 +3345,7 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr"/>
@@ -3357,7 +3361,7 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr"/>
@@ -3373,14 +3377,14 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B106" s="13" t="inlineStr">
         <is>
@@ -3389,14 +3393,14 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B107" s="13" t="inlineStr">
         <is>
@@ -3405,7 +3409,7 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr"/>
@@ -3421,7 +3425,7 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr"/>
@@ -3437,14 +3441,14 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
@@ -3453,14 +3457,14 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
@@ -3469,7 +3473,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr"/>
@@ -3485,7 +3489,7 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>AI Development Context: every module: README</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr"/>
@@ -3501,7 +3505,7 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>AI Development Context: every module: ownership metadata</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr"/>
@@ -3517,7 +3521,7 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>AI Development Context: every module: dependencies</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr"/>
@@ -3533,10 +3537,42 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D115" s="11" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B116" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C116" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D116" s="11" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D115" s="11" t="inlineStr"/>
+      <c r="D117" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3552,7 +3588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4424,6 +4460,70 @@
       <c r="F27" s="11" t="inlineStr">
         <is>
           <t>Phase 22</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Generic event envelope ingestion; analytics_events is a landing buffer, never a query surface</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>analytics_events</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>Open (IP-rate-limited) to track; platform.admin-only debug listing</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Phase 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>worker: analyticspipeline</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>worker</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Claims unflushed events, batches as NDJSON, writes to MinIO/S3 - the ClickHouse/warehouse/data-lake landing pattern</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>reads/writes analytics_events; writes MinIO/S3</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="inlineStr">
+        <is>
+          <t>n/a (background)</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Phase 23</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7862,6 +7962,60 @@
       <c r="E138" s="11" t="inlineStr">
         <is>
           <t>the one route on this platform with no requireUser/requireActive</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>/v1/analytics/events</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr">
+        <is>
+          <t>Open (IP-rate-limited, no Bearer token)</t>
+        </is>
+      </c>
+      <c r="E139" s="11" t="inlineStr">
+        <is>
+          <t>the platform's one deliberately unauthenticated write endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B140" s="11" t="inlineStr">
+        <is>
+          <t>/v1/analytics/events</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>analytics</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>platform.admin</t>
+        </is>
+      </c>
+      <c r="E140" s="11" t="inlineStr">
+        <is>
+          <t>operational debug view only, not for analytical queries</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 24
Roadmap/Todo/Modules/API Endpoints/Infra sheets updated for AI Gateway
(3 routes, 142 total endpoints, a new Ollama infra row, 32 commits,
61/122 todo items done).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D117" headerRowCount="1">
-  <autoFilter ref="A1:D117"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D123" headerRowCount="1">
+  <autoFilter ref="A1:D123"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -252,8 +252,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F29" headerRowCount="1">
-  <autoFilter ref="A1:F29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Modules" displayName="Modules" ref="A1:F31" headerRowCount="1">
+  <autoFilter ref="A1:F31"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Module"/>
     <tableColumn id="2" name="Service"/>
@@ -267,8 +267,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E140" headerRowCount="1">
-  <autoFilter ref="A1:E140"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="APIEndpoints" displayName="APIEndpoints" ref="A1:E143" headerRowCount="1">
+  <autoFilter ref="A1:E143"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Method"/>
     <tableColumn id="2" name="Path"/>
@@ -294,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InfraCredentials" displayName="InfraCredentials" ref="A1:E13" headerRowCount="1">
-  <autoFilter ref="A1:E13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InfraCredentials" displayName="InfraCredentials" ref="A1:E14" headerRowCount="1">
+  <autoFilter ref="A1:E14"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Service"/>
     <tableColumn id="2" name="Type"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>23 / 30</t>
+          <t>24 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>77%</t>
+          <t>80%</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>142</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0021</t>
+          <t>data/migrations/0001-0022</t>
         </is>
       </c>
     </row>
@@ -735,12 +735,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, OTel</t>
+          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, Ollama, OTel</t>
         </is>
       </c>
     </row>
@@ -752,7 +752,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1446,9 +1446,9 @@
       <c r="A25" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -1458,12 +1458,12 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>Provider-neutral interface (OpenAI/Anthropic/Google/local models/Ollama/vLLM) with model routing, quotas, token/cost tracking, audit, timeouts, fallback. Products never call AI vendors directly.</t>
+          <t>Provider-neutral interface; real local inference via a new Ollama container (auto-pulled model, no vendor API key) - the one live-testable provider. Model routing, quotas (ratelimit reused again), real token/cost tracking, a genuine audit.Record per call, prompt/version metadata, timeouts, fallback. OpenAI/Anthropic/Google structurally supported, not implemented (no real credentials).</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>d7324b9</t>
         </is>
       </c>
     </row>
@@ -1471,9 +1471,9 @@
       <c r="A26" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2032,7 +2032,7 @@
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
@@ -2041,14 +2041,14 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 24: AI Gateway implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
@@ -2057,18 +2057,14 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
@@ -2077,32 +2073,32 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2117,12 +2113,12 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2137,30 +2133,34 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B31" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr"/>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr"/>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr"/>
@@ -2246,21 +2246,17 @@
       <c r="A37" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B37" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D37" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="9" t="n">
@@ -2273,32 +2269,32 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2313,10 +2309,14 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
@@ -2345,7 +2345,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
@@ -2466,21 +2466,17 @@
       <c r="A50" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
@@ -2493,30 +2489,34 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>21</v>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Billing: Payment model (provider-specific transaction record)</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr"/>
@@ -2561,32 +2561,28 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Billing: Stripe adapter</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="inlineStr">
-        <is>
-          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
-        </is>
-      </c>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Billing: Apple IAP adapter</t>
+          <t>Billing: Stripe adapter</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
         </is>
       </c>
     </row>
@@ -2601,30 +2597,34 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Billing: Google Play adapter</t>
+          <t>Billing: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>22</v>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
+          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr"/>
@@ -2662,25 +2662,21 @@
       <c r="A61" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="inlineStr">
-        <is>
-          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
-        </is>
-      </c>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B62" s="13" t="inlineStr">
         <is>
@@ -2689,23 +2685,27 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (OpenAI/Anthropic/Google/local/Ollama/vLLM)</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr"/>
+          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing</t>
+          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
@@ -2714,17 +2714,21 @@
       <c r="A64" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr"/>
+          <t>AI Gateway: local models / Ollama adapter</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
@@ -2737,10 +2741,14 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="inlineStr"/>
+          <t>AI Gateway: OpenAI adapter</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
@@ -2753,10 +2761,14 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="inlineStr"/>
+          <t>AI Gateway: Anthropic adapter</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -2769,23 +2781,27 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="inlineStr"/>
+          <t>AI Gateway: Google adapter</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B68" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata</t>
+          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr"/>
@@ -2794,14 +2810,14 @@
       <c r="A69" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts</t>
+          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr"/>
@@ -2810,101 +2826,101 @@
       <c r="A70" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B70" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>24</v>
+      </c>
+      <c r="B71" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: control-plane UI in apps/admin</t>
+          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>24</v>
+      </c>
+      <c r="B72" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Applications</t>
+          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>24</v>
+      </c>
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
+          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>24</v>
+      </c>
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Roles/Permissions</t>
+          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B75" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>24</v>
+      </c>
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Tenants/Relationships</t>
+          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="9" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
@@ -2913,10 +2929,14 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Messages/Notifications</t>
-        </is>
-      </c>
-      <c r="D76" s="11" t="inlineStr"/>
+          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
+        </is>
+      </c>
+      <c r="D76" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
@@ -2929,7 +2949,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Files/Jobs</t>
+          <t>Admin Portal: control-plane UI in apps/admin</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
@@ -2945,7 +2965,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Feature flags/Configuration</t>
+          <t>Admin Portal: visibility: Applications</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
@@ -2961,7 +2981,7 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: Moderation/Audit</t>
+          <t>Admin Portal: visibility: Users/Sessions/Devices</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr"/>
@@ -2977,7 +2997,7 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility: System health/Deployments</t>
+          <t>Admin Portal: visibility: Roles/Permissions</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr"/>
@@ -2993,14 +3013,14 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
+          <t>Admin Portal: visibility: Tenants/Relationships</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B82" s="13" t="inlineStr">
         <is>
@@ -3009,14 +3029,14 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: visibility: Messages/Notifications</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B83" s="13" t="inlineStr">
         <is>
@@ -3025,14 +3045,14 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
+          <t>Admin Portal: visibility: Files/Jobs</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B84" s="13" t="inlineStr">
         <is>
@@ -3041,14 +3061,14 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
+          <t>Admin Portal: visibility: Feature flags/Configuration</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B85" s="13" t="inlineStr">
         <is>
@@ -3057,14 +3077,14 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
+          <t>Admin Portal: visibility: Moderation/Audit</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
@@ -3073,14 +3093,14 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
+          <t>Admin Portal: visibility: System health/Deployments</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B87" s="13" t="inlineStr">
         <is>
@@ -3089,14 +3109,14 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
+          <t>Admin Portal: must go through service APIs, never direct DB queries</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
@@ -3105,14 +3125,14 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B89" s="13" t="inlineStr">
         <is>
@@ -3121,14 +3141,14 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
+          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B90" s="13" t="inlineStr">
         <is>
@@ -3137,14 +3157,14 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
+          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B91" s="13" t="inlineStr">
         <is>
@@ -3153,7 +3173,7 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
+          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr"/>
@@ -3169,7 +3189,7 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: Flutter SDK</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr"/>
@@ -3185,14 +3205,14 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B94" s="13" t="inlineStr">
         <is>
@@ -3201,14 +3221,14 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
@@ -3217,14 +3237,14 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B96" s="13" t="inlineStr">
         <is>
@@ -3233,14 +3253,14 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B97" s="13" t="inlineStr">
         <is>
@@ -3249,14 +3269,14 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
@@ -3265,14 +3285,14 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B99" s="13" t="inlineStr">
         <is>
@@ -3281,7 +3301,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr"/>
@@ -3297,7 +3317,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr"/>
@@ -3313,7 +3333,7 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr"/>
@@ -3329,7 +3349,7 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr"/>
@@ -3345,7 +3365,7 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr"/>
@@ -3361,7 +3381,7 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr"/>
@@ -3377,7 +3397,7 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr"/>
@@ -3393,7 +3413,7 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr"/>
@@ -3409,14 +3429,14 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
@@ -3425,14 +3445,14 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B109" s="13" t="inlineStr">
         <is>
@@ -3441,14 +3461,14 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B110" s="13" t="inlineStr">
         <is>
@@ -3457,14 +3477,14 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B111" s="13" t="inlineStr">
         <is>
@@ -3473,14 +3493,14 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B112" s="13" t="inlineStr">
         <is>
@@ -3489,14 +3509,14 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B113" s="13" t="inlineStr">
         <is>
@@ -3505,14 +3525,14 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
@@ -3521,14 +3541,14 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
@@ -3537,14 +3557,14 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
@@ -3553,26 +3573,122 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B117" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+        </is>
+      </c>
+      <c r="D117" s="11" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B117" s="13" t="inlineStr">
+      <c r="B118" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C117" s="11" t="inlineStr">
+      <c r="C118" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: README</t>
+        </is>
+      </c>
+      <c r="D118" s="11" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: ownership metadata</t>
+        </is>
+      </c>
+      <c r="D119" s="11" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B120" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C120" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: dependencies</t>
+        </is>
+      </c>
+      <c r="D120" s="11" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B121" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C121" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D121" s="11" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B122" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C122" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D122" s="11" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
         <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D117" s="11" t="inlineStr"/>
+      <c r="D123" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3588,7 +3704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4524,6 +4640,70 @@
       <c r="F29" s="11" t="inlineStr">
         <is>
           <t>Phase 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>aigateway</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Provider-neutral completions API - model routing, quotas, cost tracking, audit, timeouts, fallback</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>ai_completions</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Self for own usage; open (quota-limited) to complete</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Phase 24</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>aigateway/ollama</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>core-api</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Real local-inference Provider adapter - the one live-testable Provider this phase ships</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>none (stateless HTTP client to a real Ollama container)</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>n/a (internal provider adapter, not a route)</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Phase 24</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E140"/>
+  <dimension ref="A1:E143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8016,6 +8196,87 @@
       <c r="E140" s="11" t="inlineStr">
         <is>
           <t>operational debug view only, not for analytical queries</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B141" s="11" t="inlineStr">
+        <is>
+          <t>/v1/ai/completions</t>
+        </is>
+      </c>
+      <c r="C141" s="11" t="inlineStr">
+        <is>
+          <t>aigateway</t>
+        </is>
+      </c>
+      <c r="D141" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated (quota-limited)</t>
+        </is>
+      </c>
+      <c r="E141" s="11" t="inlineStr">
+        <is>
+          <t>real local inference via Ollama; never call a vendor model name directly</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B142" s="11" t="inlineStr">
+        <is>
+          <t>/v1/ai/usage</t>
+        </is>
+      </c>
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>aigateway</t>
+        </is>
+      </c>
+      <c r="D142" s="11" t="inlineStr">
+        <is>
+          <t>Self or platform.admin</t>
+        </is>
+      </c>
+      <c r="E142" s="11" t="inlineStr">
+        <is>
+          <t>?userId=; tokens/cost/latency, never prompt or response text</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="11" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>/v1/ai/models</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="inlineStr">
+        <is>
+          <t>aigateway</t>
+        </is>
+      </c>
+      <c r="D143" s="11" t="inlineStr">
+        <is>
+          <t>Authenticated</t>
+        </is>
+      </c>
+      <c r="E143" s="11" t="inlineStr">
+        <is>
+          <t>lists registered model aliases, never vendor model names</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -8583,7 +8844,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Background job runner, search indexer, Temporal workflow worker.</t>
+          <t>Background job runner, search indexer, Temporal workflow worker, analytics NDJSON pipeline.</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -8811,25 +9072,52 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Docker container</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>http://localhost:11434</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Real local LLM inference behind the AI Gateway - model qwen2.5:0.5b auto-pulled on every start, no vendor API key needed.</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>no auth locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
           <t>OTel Collector / Tempo / Prometheus / Grafana / Loki</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Docker containers</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>see infra/docker/docker-compose.yml</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>Full observability stack - traces, metrics, logs, dashboards.</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>no auth locally</t>
         </is>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 26
Roadmap/Todo/Stats/Infra/How-To-Test sheets updated for the Backstage
phase: Phase 26 marked Done with its real commit hash, Phase 27 (SDKs)
promoted to Next up, a new Infra & Credentials row for platform/
backstage (noting its port collision with apps/admin), and a How To
Test step for browsing the real catalog.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D123" headerRowCount="1">
-  <autoFilter ref="A1:D123"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D129" headerRowCount="1">
+  <autoFilter ref="A1:D129"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -281,8 +281,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D20" headerRowCount="1">
-  <autoFilter ref="A1:D20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D21" headerRowCount="1">
+  <autoFilter ref="A1:D21"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Step"/>
     <tableColumn id="2" name="What"/>
@@ -294,8 +294,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InfraCredentials" displayName="InfraCredentials" ref="A1:E15" headerRowCount="1">
-  <autoFilter ref="A1:E15"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="InfraCredentials" displayName="InfraCredentials" ref="A1:E16" headerRowCount="1">
+  <autoFilter ref="A1:E16"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Service"/>
     <tableColumn id="2" name="Type"/>
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>25 / 30</t>
+          <t>26 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>83%</t>
+          <t>87%</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Shared Go packages</t>
+          <t>Developer portal</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -689,139 +689,156 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>packages/go/platformkit</t>
+          <t>platform/backstage (real @backstage/create-app, 24-entity catalog)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Domain modules (core-api)</t>
+          <t>Shared Go packages</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>one per completed backend phase</t>
+          <t>packages/go/platformkit</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Live HTTP endpoints</t>
+          <t>Domain modules (core-api)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>see 'API Endpoints' sheet</t>
+          <t>one per completed backend phase</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>DB migrations</t>
+          <t>Live HTTP endpoints</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>146</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0022</t>
+          <t>see 'API Endpoints' sheet</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Real infra dependencies</t>
+          <t>DB migrations</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, Ollama, OTel</t>
+          <t>data/migrations/0001-0022</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>Real infra dependencies</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, Ollama, OTel</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>Commits so far</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>see git log</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>• Roadmap - all 30 phases, one row each, status + what it delivers.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>• Todo Checklist - granular task list (completed sub-items and still-to-do sub-items) so progress is trackable at a finer grain than 'phase done or not'.</t>
+          <t>• Roadmap - all 30 phases, one row each, status + what it delivers.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>• Modules - every backend/core-api/internal module: what it owns, its storage, its access rule.</t>
+          <t>• Todo Checklist - granular task list (completed sub-items and still-to-do sub-items) so progress is trackable at a finer grain than 'phase done or not'.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>• API Endpoints - every live HTTP route across all three services, with auth level.</t>
+          <t>• Modules - every backend/core-api/internal module: what it owns, its storage, its access rule.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>• How To Test - copy-paste steps to bring the stack up locally and exercise it for real (mint a token, call endpoints, open a WebSocket).</t>
+          <t>• API Endpoints - every live HTTP route across all three services, with auth level.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>• How To Test - copy-paste steps to bring the stack up locally and exercise it for real (mint a token, call endpoints, open a WebSocket).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>• Infra &amp; Credentials - every local service, its port, and its local-only credentials.</t>
         </is>
@@ -830,8 +847,8 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A20:F20"/>
@@ -1513,9 +1530,9 @@
       <c r="A27" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
@@ -1525,12 +1542,12 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>Integrate Backstage as the developer portal - every service/module exposes metadata (owner, lifecycle, repo, docs, dependencies, APIs, events, DB ownership, dashboards, runbooks). Backstage becomes the map of the platform.</t>
+          <t>A real @backstage/create-app instance (platform/backstage) whose catalog (catalog/system.yaml) is 24 real entities - a Group, the System, Components for all 3 services + admin + 16 domain modules with real dependsOn/providesApis, and 2 API entities embedding the full real OpenAPI/AsyncAPI specs. Filled in 11 stub module READMEs, fixed 2 real YAML bugs in the OpenAPI spec, generated ~110 missing OpenAPI paths from the actual Go route registrations, and live-validated the whole catalog loads with zero processing errors via the real catalog API.</t>
         </is>
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>b1bf7b9</t>
         </is>
       </c>
     </row>
@@ -1538,9 +1555,9 @@
       <c r="A28" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -1648,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2081,7 +2098,7 @@
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
@@ -2090,14 +2107,14 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 26: Backstage implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
@@ -2106,18 +2123,14 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
@@ -2126,32 +2139,32 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2179,12 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2186,30 +2199,34 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B33" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D33" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
@@ -2222,7 +2239,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr"/>
@@ -2238,7 +2255,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
@@ -2254,7 +2271,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr"/>
@@ -2270,7 +2287,7 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr"/>
@@ -2286,7 +2303,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
@@ -2295,21 +2312,17 @@
       <c r="A39" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="n">
@@ -2322,32 +2335,32 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2362,10 +2375,14 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -2378,7 +2395,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr"/>
@@ -2394,7 +2411,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2410,7 +2427,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2426,7 +2443,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2442,7 +2459,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2458,7 +2475,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
@@ -2474,7 +2491,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
@@ -2490,7 +2507,7 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
@@ -2506,7 +2523,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr"/>
@@ -2515,21 +2532,17 @@
       <c r="A52" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
@@ -2542,30 +2555,34 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B54" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>21</v>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Billing: Payment model (provider-specific transaction record)</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
@@ -2578,7 +2595,7 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr"/>
@@ -2594,7 +2611,7 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr"/>
@@ -2610,32 +2627,28 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Billing: Stripe adapter</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="inlineStr">
-        <is>
-          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
-        </is>
-      </c>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Billing: Apple IAP adapter</t>
+          <t>Billing: Stripe adapter</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
         </is>
       </c>
     </row>
@@ -2650,30 +2663,34 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Billing: Google Play adapter</t>
+          <t>Billing: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>22</v>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
@@ -2686,7 +2703,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
+          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr"/>
@@ -2702,7 +2719,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
@@ -2711,37 +2728,37 @@
       <c r="A63" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="inlineStr">
-        <is>
-          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
-        </is>
-      </c>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>23</v>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr"/>
+          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
@@ -2754,32 +2771,28 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: local models / Ollama adapter</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="inlineStr">
-        <is>
-          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
-        </is>
-      </c>
+          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: OpenAI adapter</t>
+          <t>AI Gateway: local models / Ollama adapter</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no real API key in this environment to validate against honestly</t>
+          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2807,7 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Anthropic adapter</t>
+          <t>AI Gateway: OpenAI adapter</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
@@ -2814,7 +2827,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Google adapter</t>
+          <t>AI Gateway: Anthropic adapter</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
@@ -2827,17 +2840,21 @@
       <c r="A69" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B69" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
-        </is>
-      </c>
-      <c r="D69" s="11" t="inlineStr"/>
+          <t>AI Gateway: Google adapter</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="n">
@@ -2850,7 +2867,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
+          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr"/>
@@ -2866,7 +2883,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
@@ -2882,7 +2899,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
@@ -2898,7 +2915,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
+          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2914,7 +2931,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
+          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2930,7 +2947,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
+          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
@@ -2946,7 +2963,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
@@ -2955,37 +2972,37 @@
       <c r="A77" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
-        </is>
-      </c>
-      <c r="D77" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
-        </is>
-      </c>
+          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+        </is>
+      </c>
+      <c r="D77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B78" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>24</v>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
-        </is>
-      </c>
-      <c r="D78" s="11" t="inlineStr"/>
+          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
@@ -2998,14 +3015,10 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Applications</t>
-        </is>
-      </c>
-      <c r="D79" s="11" t="inlineStr">
-        <is>
-          <t>Real GET /v1/apps table</t>
-        </is>
-      </c>
+          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n">
@@ -3018,12 +3031,12 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Users (list + detail)</t>
+          <t>Admin Portal: visibility - Applications</t>
         </is>
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
+          <t>Real GET /v1/apps table</t>
         </is>
       </c>
     </row>
@@ -3038,12 +3051,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Roles/Permissions</t>
+          <t>Admin Portal: visibility - Users (list + detail)</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
         </is>
       </c>
     </row>
@@ -3058,10 +3071,14 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
-        </is>
-      </c>
-      <c r="D82" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - Roles/Permissions</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr">
+        <is>
+          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
@@ -3074,7 +3091,7 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Moderation, Audit</t>
+          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr"/>
@@ -3090,14 +3107,10 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - System Health</t>
-        </is>
-      </c>
-      <c r="D84" s="11" t="inlineStr">
-        <is>
-          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Moderation, Audit</t>
+        </is>
+      </c>
+      <c r="D84" s="11" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
@@ -3110,30 +3123,30 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
-        </is>
-      </c>
-      <c r="D85" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - System Health</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B86" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
-        </is>
-      </c>
-      <c r="D86" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n">
@@ -3146,18 +3159,18 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Deployments</t>
+          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
+          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
@@ -3166,110 +3179,138 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
-        </is>
-      </c>
-      <c r="D88" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - Deployments</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: name/description/owner/lifecycle</t>
-        </is>
-      </c>
-      <c r="D89" s="11" t="inlineStr"/>
+          <t>Backstage: integrate Backstage as developer portal</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr">
+        <is>
+          <t>Real @backstage/create-app instance at platform/backstage, catalog wired to real catalog/*.yaml + contracts/*/catalog-info.yaml, live-validated via the real catalog API (21 Components, 2 APIs, 1 System, 1 Group, 0 processing errors)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B90" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: repository/documentation/dependencies</t>
-        </is>
-      </c>
-      <c r="D90" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - name/description/owner/lifecycle</t>
+        </is>
+      </c>
+      <c r="D90" s="11" t="inlineStr">
+        <is>
+          <t>All 16 modules/*/module.yaml + README.md real (11 were still stub text before this phase)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B91" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B91" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata: APIs/events/DB ownership/dashboards/runbooks</t>
-        </is>
-      </c>
-      <c r="D91" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - repository/documentation</t>
+        </is>
+      </c>
+      <c r="D91" s="11" t="inlineStr">
+        <is>
+          <t>Every Component links its module README; the System entity links VALIDATION.md and the new docs/RUNBOOKS.md</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B92" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B92" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
-        </is>
-      </c>
-      <c r="D92" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - dependencies</t>
+        </is>
+      </c>
+      <c r="D92" s="11" t="inlineStr">
+        <is>
+          <t>Component dependsOn mirrors modules/*/module.yaml's real dependency graph; Backstage computes reverse dependencyOf relations automatically, confirmed live</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B93" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B93" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
-        </is>
-      </c>
-      <c r="D93" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - APIs</t>
+        </is>
+      </c>
+      <c r="D93" s="11" t="inlineStr">
+        <is>
+          <t>2 API entities (OpenAPI, AsyncAPI), both with their full real spec embedded and live-loaded</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B94" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B94" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
-        </is>
-      </c>
-      <c r="D94" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - events</t>
+        </is>
+      </c>
+      <c r="D94" s="11" t="inlineStr">
+        <is>
+          <t>providesApis set only on the components whose code actually calls outbox.Record, cross-checked against the real Go source</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B95" s="13" t="inlineStr">
         <is>
@@ -3278,42 +3319,54 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
-        </is>
-      </c>
-      <c r="D95" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - database ownership</t>
+        </is>
+      </c>
+      <c r="D95" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no per-module DB-ownership annotation convention chosen yet; docs/control's Modules sheet tracks this today at a finer grain than catalog/system.yaml's 16 domains</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B96" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B96" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
-        </is>
-      </c>
-      <c r="D96" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - dashboards</t>
+        </is>
+      </c>
+      <c r="D96" s="11" t="inlineStr">
+        <is>
+          <t>core-platform.io/dashboard annotation on each service pointing at the real local Grafana instance - no per-service dashboard exists yet (that's Phase 28), so it points at the shared instance, documented as such</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
-        </is>
-      </c>
-      <c r="D97" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - runbooks</t>
+        </is>
+      </c>
+      <c r="D97" s="11" t="inlineStr">
+        <is>
+          <t>New docs/RUNBOOKS.md, linked from the System entity</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n">
@@ -3326,7 +3379,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: Flutter SDK</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr"/>
@@ -3342,14 +3395,14 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B100" s="13" t="inlineStr">
         <is>
@@ -3358,14 +3411,14 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B101" s="13" t="inlineStr">
         <is>
@@ -3374,14 +3427,14 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B102" s="13" t="inlineStr">
         <is>
@@ -3390,14 +3443,14 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B103" s="13" t="inlineStr">
         <is>
@@ -3406,14 +3459,14 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B104" s="13" t="inlineStr">
         <is>
@@ -3422,14 +3475,14 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B105" s="13" t="inlineStr">
         <is>
@@ -3438,7 +3491,7 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr"/>
@@ -3454,7 +3507,7 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr"/>
@@ -3470,7 +3523,7 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr"/>
@@ -3486,7 +3539,7 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr"/>
@@ -3502,7 +3555,7 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
@@ -3518,7 +3571,7 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
@@ -3534,7 +3587,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr"/>
@@ -3550,7 +3603,7 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr"/>
@@ -3566,14 +3619,14 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B114" s="13" t="inlineStr">
         <is>
@@ -3582,14 +3635,14 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B115" s="13" t="inlineStr">
         <is>
@@ -3598,14 +3651,14 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B116" s="13" t="inlineStr">
         <is>
@@ -3614,14 +3667,14 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B117" s="13" t="inlineStr">
         <is>
@@ -3630,14 +3683,14 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B118" s="13" t="inlineStr">
         <is>
@@ -3646,14 +3699,14 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="9" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B119" s="13" t="inlineStr">
         <is>
@@ -3662,14 +3715,14 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
@@ -3678,14 +3731,14 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
@@ -3694,14 +3747,14 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
@@ -3710,26 +3763,122 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B123" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+        </is>
+      </c>
+      <c r="D123" s="11" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B123" s="13" t="inlineStr">
+      <c r="B124" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C123" s="11" t="inlineStr">
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: README</t>
+        </is>
+      </c>
+      <c r="D124" s="11" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B125" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: ownership metadata</t>
+        </is>
+      </c>
+      <c r="D125" s="11" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B126" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: dependencies</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B127" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D127" s="11" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B129" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
         <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D123" s="11" t="inlineStr"/>
+      <c r="D129" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8443,7 +8592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8889,6 +9038,28 @@
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Then open http://localhost:3000 and sign in with demo/demo. Real UI over real data (Phase 25) - Users, Roles, Audit, Moderation, Feature Flags, Jobs, Configuration, System Health, Billing, AI Gateway. Needs core-api (and ideally realtime-gateway/worker) already running per steps 5-7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Browse the real developer-portal catalog</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>cd platform/backstage &amp;&amp; yarn install &amp;&amp; yarn start</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Needs Node 20/22 and a real Yarn install - see platform/backstage/README.md if the versions on $PATH don't satisfy Backstage's own prerequisite check. Then open http://localhost:3000 (stop the Admin Portal first, they share a port) and browse the Catalog - every module/service/app is a real entity (Phase 26), not example fixture data.</t>
         </is>
       </c>
     </row>
@@ -8906,7 +9077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -9000,34 +9171,34 @@
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>realtime-gateway</t>
+          <t>backstage (platform/backstage)</t>
         </is>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>Go service</t>
+          <t>Backstage app</t>
         </is>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>ws://localhost:8090</t>
+          <t>http://localhost:3000 (frontend), :7007 (backend)</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>WebSocket connections, presence, channel fan-out.</t>
+          <t>The developer portal (Phase 26) - real catalog of every module/service/app. Shares apps/admin's default frontend port 3000, so only run one of the two at a time locally unless one's app-config.yaml is repointed at a different port.</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>guest auth only, no credentials</t>
         </is>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>worker</t>
+          <t>realtime-gateway</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -9037,12 +9208,12 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:8091 (health only)</t>
+          <t>ws://localhost:8090</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>Background job runner, search indexer, Temporal workflow worker, analytics NDJSON pipeline.</t>
+          <t>WebSocket connections, presence, channel fan-out.</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -9054,34 +9225,34 @@
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Postgres</t>
+          <t>worker</t>
         </is>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Docker container</t>
+          <t>Go service</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>localhost:5432</t>
+          <t>http://localhost:8091 (health only)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>System of record for every domain module.</t>
+          <t>Background job runner, search indexer, Temporal workflow worker, analytics NDJSON pipeline.</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>core / core, db 'core'</t>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Valkey (Redis-compatible)</t>
+          <t>Postgres</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
@@ -9091,24 +9262,24 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>localhost:6379</t>
+          <t>localhost:5432</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Realtime pub/sub fan-out, presence (TTL-based).</t>
+          <t>System of record for every domain module.</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>no auth locally</t>
+          <t>core / core, db 'core'</t>
         </is>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Keycloak</t>
+          <t>Valkey (Redis-compatible)</t>
         </is>
       </c>
       <c r="B8" s="11" t="inlineStr">
@@ -9118,24 +9289,24 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:8081</t>
+          <t>localhost:6379</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Identity provider. Realm 'core' is re-imported on every restart (no persistent volume).</t>
+          <t>Realtime pub/sub fan-out, presence (TTL-based).</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>admin/admin (master realm); demo/demo (core realm, seeded user)</t>
+          <t>no auth locally</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>OpenFGA</t>
+          <t>Keycloak</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
@@ -9145,24 +9316,24 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:8082</t>
+          <t>http://localhost:8081</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>Fine-grained ReBAC engine behind authz.Service.Can. In-memory store, self-heals its store/model on every restart.</t>
+          <t>Identity provider. Realm 'core' is re-imported on every restart (no persistent volume).</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>no auth locally</t>
+          <t>admin/admin (master realm); demo/demo (core realm, seeded user)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>MinIO (S3-compatible)</t>
+          <t>OpenFGA</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">
@@ -9172,24 +9343,24 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:9000</t>
+          <t>http://localhost:8082</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Object storage backing the files module.</t>
+          <t>Fine-grained ReBAC engine behind authz.Service.Can. In-memory store, self-heals its store/model on every restart.</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>minio / minio123, bucket 'core-platform'</t>
+          <t>no auth locally</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>OpenSearch</t>
+          <t>MinIO (S3-compatible)</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
@@ -9199,24 +9370,24 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:9200</t>
+          <t>http://localhost:9000</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>Backs the search module, indexed by worker's indexer.</t>
+          <t>Object storage backing the files module.</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>no auth locally</t>
+          <t>minio / minio123, bucket 'core-platform'</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Temporal</t>
+          <t>OpenSearch</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
@@ -9226,12 +9397,12 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>localhost:7233</t>
+          <t>http://localhost:9200</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Durable workflow execution engine behind the workflows module.</t>
+          <t>Backs the search module, indexed by worker's indexer.</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
@@ -9243,7 +9414,7 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Kafka / Redpanda</t>
+          <t>Temporal</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
@@ -9253,12 +9424,12 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>localhost:9092</t>
+          <t>localhost:7233</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Health-checked today; no producer wired yet (outbox-to-Kafka relay is a documented future gap).</t>
+          <t>Durable workflow execution engine behind the workflows module.</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -9270,7 +9441,7 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Ollama</t>
+          <t>Kafka / Redpanda</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -9280,12 +9451,12 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>http://localhost:11434</t>
+          <t>localhost:9092</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Real local LLM inference behind the AI Gateway - model qwen2.5:0.5b auto-pulled on every start, no vendor API key needed.</t>
+          <t>Health-checked today; no producer wired yet (outbox-to-Kafka relay is a documented future gap).</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -9297,25 +9468,52 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
+          <t>Ollama</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Docker container</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>http://localhost:11434</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Real local LLM inference behind the AI Gateway - model qwen2.5:0.5b auto-pulled on every start, no vendor API key needed.</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>no auth locally</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
           <t>OTel Collector / Tempo / Prometheus / Grafana / Loki</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Docker containers</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>see infra/docker/docker-compose.yml</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Full observability stack - traces, metrics, logs, dashboards.</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>no auth locally</t>
         </is>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 27
Roadmap/Todo/Stats/How-To-Test sheets updated for the SDKs phase:
Phase 27 marked Done with its real commit hash, Phase 28
(Observability Completion) promoted to Next up, and three new How To
Test steps for running each SDK's own test suite.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D129" headerRowCount="1">
-  <autoFilter ref="A1:D129"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D132" headerRowCount="1">
+  <autoFilter ref="A1:D132"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -281,8 +281,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D21" headerRowCount="1">
-  <autoFilter ref="A1:D21"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D24" headerRowCount="1">
+  <autoFilter ref="A1:D24"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Step"/>
     <tableColumn id="2" name="What"/>
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>26 / 30</t>
+          <t>27 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>87%</t>
+          <t>90%</t>
         </is>
       </c>
     </row>
@@ -689,156 +689,173 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>platform/backstage (real @backstage/create-app, 24-entity catalog)</t>
+          <t>platform/backstage (real @backstage/create-app, 27-entity catalog)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Shared Go packages</t>
+          <t>Client SDKs</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>packages/go/platformkit</t>
+          <t>Go, TypeScript, Dart - packages/go/coresdk, packages/typescript/core-sdk, packages/flutter/core_sdk</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Domain modules (core-api)</t>
+          <t>Shared Go packages</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>one per completed backend phase</t>
+          <t>packages/go/platformkit</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Live HTTP endpoints</t>
+          <t>Domain modules (core-api)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>146</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>see 'API Endpoints' sheet</t>
+          <t>one per completed backend phase</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>DB migrations</t>
+          <t>Live HTTP endpoints</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>146</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>data/migrations/0001-0022</t>
+          <t>see 'API Endpoints' sheet</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Real infra dependencies</t>
+          <t>DB migrations</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, Ollama, OTel</t>
+          <t>data/migrations/0001-0022</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>Real infra dependencies</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Postgres, Valkey, Keycloak, OpenFGA, MinIO, OpenSearch, Temporal, Kafka/Redpanda, Ollama, OTel</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Commits so far</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>see git log</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>How to read this workbook</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>• Roadmap - all 30 phases, one row each, status + what it delivers.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>• Todo Checklist - granular task list (completed sub-items and still-to-do sub-items) so progress is trackable at a finer grain than 'phase done or not'.</t>
+          <t>• Roadmap - all 30 phases, one row each, status + what it delivers.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>• Modules - every backend/core-api/internal module: what it owns, its storage, its access rule.</t>
+          <t>• Todo Checklist - granular task list (completed sub-items and still-to-do sub-items) so progress is trackable at a finer grain than 'phase done or not'.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>• API Endpoints - every live HTTP route across all three services, with auth level.</t>
+          <t>• Modules - every backend/core-api/internal module: what it owns, its storage, its access rule.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>• How To Test - copy-paste steps to bring the stack up locally and exercise it for real (mint a token, call endpoints, open a WebSocket).</t>
+          <t>• API Endpoints - every live HTTP route across all three services, with auth level.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>• How To Test - copy-paste steps to bring the stack up locally and exercise it for real (mint a token, call endpoints, open a WebSocket).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>• Infra &amp; Credentials - every local service, its port, and its local-only credentials.</t>
         </is>
@@ -848,8 +865,8 @@
   <mergeCells count="7">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A21:F21"/>
@@ -1555,9 +1572,9 @@
       <c r="A28" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
@@ -1567,12 +1584,12 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Flutter SDK, TypeScript SDK, Go SDK - auth, token refresh, API calls, errors, pagination, safe retries, realtime connection, correlation IDs, device registration. Future products talk to Core primarily through these.</t>
+          <t>Go (packages/go/coresdk), TypeScript (packages/typescript/core-sdk), and Dart (packages/flutter/core_sdk) - auth/token refresh, typed API calls, errors, pagination, GET-only retries, a real realtime WebSocket client, device registration, in all three. Each proven by a real consumer: apps/admin migrated its entire API layer to the TS SDK; apps/mobile's login/profile flow uses the Dart SDK (and closed a real Phase 9 gap - make flutter-test now passes). 39 unit tests total, all against real local HTTP servers, plus live validation against real Keycloak/core-api/realtime-gateway for all three.</t>
         </is>
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12b9046</t>
         </is>
       </c>
     </row>
@@ -1580,9 +1597,9 @@
       <c r="A29" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -1665,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2114,7 +2131,7 @@
     </row>
     <row r="28">
       <c r="A28" s="9" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
@@ -2123,14 +2140,14 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 27: SDKs implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
@@ -2139,18 +2156,14 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
@@ -2159,32 +2172,32 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2199,12 +2212,12 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2219,30 +2232,34 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B34" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
@@ -2255,7 +2272,7 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr"/>
@@ -2271,7 +2288,7 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr"/>
@@ -2287,7 +2304,7 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr"/>
@@ -2303,7 +2320,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
@@ -2319,7 +2336,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
@@ -2328,21 +2345,17 @@
       <c r="A40" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B40" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
@@ -2355,32 +2368,32 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2395,10 +2408,14 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D43" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
@@ -2411,7 +2428,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr"/>
@@ -2427,7 +2444,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr"/>
@@ -2443,7 +2460,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2459,7 +2476,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2475,7 +2492,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
@@ -2491,7 +2508,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
@@ -2507,7 +2524,7 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
@@ -2523,7 +2540,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr"/>
@@ -2539,7 +2556,7 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
@@ -2548,21 +2565,17 @@
       <c r="A53" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D53" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="9" t="n">
@@ -2575,30 +2588,34 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B55" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>21</v>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Billing: Payment model (provider-specific transaction record)</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
@@ -2611,7 +2628,7 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr"/>
@@ -2627,7 +2644,7 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr"/>
@@ -2643,32 +2660,28 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Billing: Stripe adapter</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
-        </is>
-      </c>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Billing: Apple IAP adapter</t>
+          <t>Billing: Stripe adapter</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
         </is>
       </c>
     </row>
@@ -2683,30 +2696,34 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Billing: Google Play adapter</t>
+          <t>Billing: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B61" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>22</v>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D61" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="n">
@@ -2719,7 +2736,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
+          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr"/>
@@ -2735,7 +2752,7 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
         </is>
       </c>
       <c r="D63" s="11" t="inlineStr"/>
@@ -2744,37 +2761,37 @@
       <c r="A64" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
-        <is>
-          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
-        </is>
-      </c>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B65" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>23</v>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
-        </is>
-      </c>
-      <c r="D65" s="11" t="inlineStr"/>
+          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
@@ -2787,32 +2804,28 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: local models / Ollama adapter</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="inlineStr">
-        <is>
-          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
-        </is>
-      </c>
+          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B67" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: OpenAI adapter</t>
+          <t>AI Gateway: local models / Ollama adapter</t>
         </is>
       </c>
       <c r="D67" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no real API key in this environment to validate against honestly</t>
+          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2840,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Anthropic adapter</t>
+          <t>AI Gateway: OpenAI adapter</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
@@ -2847,7 +2860,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Google adapter</t>
+          <t>AI Gateway: Anthropic adapter</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
@@ -2860,17 +2873,21 @@
       <c r="A70" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B70" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
-        </is>
-      </c>
-      <c r="D70" s="11" t="inlineStr"/>
+          <t>AI Gateway: Google adapter</t>
+        </is>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
@@ -2883,7 +2900,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
+          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr"/>
@@ -2899,7 +2916,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
         </is>
       </c>
       <c r="D72" s="11" t="inlineStr"/>
@@ -2915,7 +2932,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2931,7 +2948,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
+          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2947,7 +2964,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
+          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
@@ -2963,7 +2980,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
+          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
@@ -2979,7 +2996,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
@@ -2988,37 +3005,37 @@
       <c r="A78" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
-        </is>
-      </c>
-      <c r="D78" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
-        </is>
-      </c>
+          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+        </is>
+      </c>
+      <c r="D78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B79" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>24</v>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
-        </is>
-      </c>
-      <c r="D79" s="11" t="inlineStr"/>
+          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
+        </is>
+      </c>
+      <c r="D79" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="n">
@@ -3031,14 +3048,10 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Applications</t>
-        </is>
-      </c>
-      <c r="D80" s="11" t="inlineStr">
-        <is>
-          <t>Real GET /v1/apps table</t>
-        </is>
-      </c>
+          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
@@ -3051,12 +3064,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Users (list + detail)</t>
+          <t>Admin Portal: visibility - Applications</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
+          <t>Real GET /v1/apps table</t>
         </is>
       </c>
     </row>
@@ -3071,12 +3084,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Roles/Permissions</t>
+          <t>Admin Portal: visibility - Users (list + detail)</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
         </is>
       </c>
     </row>
@@ -3091,10 +3104,14 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
-        </is>
-      </c>
-      <c r="D83" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - Roles/Permissions</t>
+        </is>
+      </c>
+      <c r="D83" s="11" t="inlineStr">
+        <is>
+          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="n">
@@ -3107,7 +3124,7 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Moderation, Audit</t>
+          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr"/>
@@ -3123,14 +3140,10 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - System Health</t>
-        </is>
-      </c>
-      <c r="D85" s="11" t="inlineStr">
-        <is>
-          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Moderation, Audit</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n">
@@ -3143,30 +3156,30 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
-        </is>
-      </c>
-      <c r="D86" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - System Health</t>
+        </is>
+      </c>
+      <c r="D86" s="11" t="inlineStr">
+        <is>
+          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B87" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B87" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
-        </is>
-      </c>
-      <c r="D87" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
@@ -3179,32 +3192,32 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Deployments</t>
+          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
         </is>
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
+          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B89" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>25</v>
+      </c>
+      <c r="B89" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: visibility - Deployments</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>Real @backstage/create-app instance at platform/backstage, catalog wired to real catalog/*.yaml + contracts/*/catalog-info.yaml, live-validated via the real catalog API (21 Components, 2 APIs, 1 System, 1 Group, 0 processing errors)</t>
+          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
         </is>
       </c>
     </row>
@@ -3219,12 +3232,12 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - name/description/owner/lifecycle</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>All 16 modules/*/module.yaml + README.md real (11 were still stub text before this phase)</t>
+          <t>Real @backstage/create-app instance at platform/backstage, catalog wired to real catalog/*.yaml + contracts/*/catalog-info.yaml, live-validated via the real catalog API (21 Components, 2 APIs, 1 System, 1 Group, 0 processing errors)</t>
         </is>
       </c>
     </row>
@@ -3239,12 +3252,12 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - repository/documentation</t>
+          <t>Backstage: per-module metadata - name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Every Component links its module README; the System entity links VALIDATION.md and the new docs/RUNBOOKS.md</t>
+          <t>All 16 modules/*/module.yaml + README.md real (11 were still stub text before this phase)</t>
         </is>
       </c>
     </row>
@@ -3259,12 +3272,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - dependencies</t>
+          <t>Backstage: per-module metadata - repository/documentation</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>Component dependsOn mirrors modules/*/module.yaml's real dependency graph; Backstage computes reverse dependencyOf relations automatically, confirmed live</t>
+          <t>Every Component links its module README; the System entity links VALIDATION.md and the new docs/RUNBOOKS.md</t>
         </is>
       </c>
     </row>
@@ -3279,12 +3292,12 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - APIs</t>
+          <t>Backstage: per-module metadata - dependencies</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>2 API entities (OpenAPI, AsyncAPI), both with their full real spec embedded and live-loaded</t>
+          <t>Component dependsOn mirrors modules/*/module.yaml's real dependency graph; Backstage computes reverse dependencyOf relations automatically, confirmed live</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3312,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - events</t>
+          <t>Backstage: per-module metadata - APIs</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>providesApis set only on the components whose code actually calls outbox.Record, cross-checked against the real Go source</t>
+          <t>2 API entities (OpenAPI, AsyncAPI), both with their full real spec embedded and live-loaded</t>
         </is>
       </c>
     </row>
@@ -3312,19 +3325,19 @@
       <c r="A95" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B95" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B95" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - database ownership</t>
+          <t>Backstage: per-module metadata - events</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no per-module DB-ownership annotation convention chosen yet; docs/control's Modules sheet tracks this today at a finer grain than catalog/system.yaml's 16 domains</t>
+          <t>providesApis set only on the components whose code actually calls outbox.Record, cross-checked against the real Go source</t>
         </is>
       </c>
     </row>
@@ -3332,19 +3345,19 @@
       <c r="A96" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B96" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B96" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - dashboards</t>
+          <t>Backstage: per-module metadata - database ownership</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>core-platform.io/dashboard annotation on each service pointing at the real local Grafana instance - no per-service dashboard exists yet (that's Phase 28), so it points at the shared instance, documented as such</t>
+          <t>Deferred - no per-module DB-ownership annotation convention chosen yet; docs/control's Modules sheet tracks this today at a finer grain than catalog/system.yaml's 16 domains</t>
         </is>
       </c>
     </row>
@@ -3359,178 +3372,218 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - runbooks</t>
+          <t>Backstage: per-module metadata - dashboards</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>New docs/RUNBOOKS.md, linked from the System entity</t>
+          <t>core-platform.io/dashboard annotation on each service pointing at the real local Grafana instance - no per-service dashboard exists yet (that's Phase 28), so it points at the shared instance, documented as such</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B98" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>26</v>
+      </c>
+      <c r="B98" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Flutter SDK</t>
-        </is>
-      </c>
-      <c r="D98" s="11" t="inlineStr"/>
+          <t>Backstage: per-module metadata - runbooks</t>
+        </is>
+      </c>
+      <c r="D98" s="11" t="inlineStr">
+        <is>
+          <t>New docs/RUNBOOKS.md, linked from the System entity</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B99" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B99" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
-        </is>
-      </c>
-      <c r="D99" s="11" t="inlineStr"/>
+          <t>SDKs: Go SDK</t>
+        </is>
+      </c>
+      <c r="D99" s="11" t="inlineStr">
+        <is>
+          <t>packages/go/coresdk - 12 unit tests (httptest.Server), live-validated against real Keycloak/core-api/realtime-gateway</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B100" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B100" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
-        </is>
-      </c>
-      <c r="D100" s="11" t="inlineStr"/>
+          <t>SDKs: TypeScript SDK</t>
+        </is>
+      </c>
+      <c r="D100" s="11" t="inlineStr">
+        <is>
+          <t>packages/typescript/core-sdk - 13 unit tests (node:http), real consumer: apps/admin's entire lib/api.ts migrated to it</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B101" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B101" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
-        </is>
-      </c>
-      <c r="D101" s="11" t="inlineStr"/>
+          <t>SDKs: Dart SDK</t>
+        </is>
+      </c>
+      <c r="D101" s="11" t="inlineStr">
+        <is>
+          <t>packages/flutter/core_sdk (pure Dart, no Flutter dependency) - 13 unit tests (dart:io HttpServer), real consumer: apps/mobile's login/profile flow</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B102" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B102" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
-        </is>
-      </c>
-      <c r="D102" s="11" t="inlineStr"/>
+          <t>SDKs: auth + token refresh in each SDK</t>
+        </is>
+      </c>
+      <c r="D102" s="11" t="inlineStr">
+        <is>
+          <t>TokenSource (static + real Keycloak password-grant with skew-aware, concurrency-coalesced refresh) in all three</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B103" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B103" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
-        </is>
-      </c>
-      <c r="D103" s="11" t="inlineStr"/>
+          <t>SDKs: pagination + safe retries</t>
+        </is>
+      </c>
+      <c r="D103" s="11" t="inlineStr">
+        <is>
+          <t>Page/paginate/collectAll over the real {items,nextCursor} shape; GET-only retries by default on transient statuses, in all three</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B104" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B104" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
-        </is>
-      </c>
-      <c r="D104" s="11" t="inlineStr"/>
+          <t>SDKs: realtime connection helper</t>
+        </is>
+      </c>
+      <c r="D104" s="11" t="inlineStr">
+        <is>
+          <t>Reproduces realtime-gateway's real ws://.../ws?access_token=&amp;deviceId= protocol and message shapes exactly, in all three - live-validated with real cross-connection fan-out</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B105" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B105" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
-        </is>
-      </c>
-      <c r="D105" s="11" t="inlineStr"/>
+          <t>SDKs: correlation ID propagation</t>
+        </is>
+      </c>
+      <c r="D105" s="11" t="inlineStr">
+        <is>
+          <t>X-Correlation-ID on every call, matching platformkit/correlation's real header name, in all three</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B106" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>27</v>
+      </c>
+      <c r="B106" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: structured logs everywhere</t>
-        </is>
-      </c>
-      <c r="D106" s="11" t="inlineStr"/>
+          <t>SDKs: device registration helper</t>
+        </is>
+      </c>
+      <c r="D106" s="11" t="inlineStr">
+        <is>
+          <t>DevicesRegister/devicesRegister in all three - realtime dial requires a real registered device id</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B107" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>27</v>
+      </c>
+      <c r="B107" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: metrics everywhere</t>
-        </is>
-      </c>
-      <c r="D107" s="11" t="inlineStr"/>
+          <t>SDKs: apps/mobile test/ directory (make flutter-test currently fails)</t>
+        </is>
+      </c>
+      <c r="D107" s="11" t="inlineStr">
+        <is>
+          <t>Closed as a side effect - real widget tests added, discovered and worked around Flutter's TestWidgetsFlutterBinding network-mocking constraint live. Was pending since Phase 9.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B108" s="13" t="inlineStr">
         <is>
@@ -3539,10 +3592,14 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: distributed traces everywhere</t>
-        </is>
-      </c>
-      <c r="D108" s="11" t="inlineStr"/>
+          <t>SDKs: full API coverage (all 146 endpoints typed) in each SDK</t>
+        </is>
+      </c>
+      <c r="D108" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - each SDK covers a representative 'core identity' slice (platform/identity/users/devices/applications) plus what its real consumer needs; the untyped request()/Do() escape hatch reaches everything else. Broader coverage is real, additive work, not a framework limitation.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="9" t="n">
@@ -3555,7 +3612,7 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: health checks everywhere</t>
+          <t>Observability Completion: structured logs everywhere</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr"/>
@@ -3571,7 +3628,7 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: API latency</t>
+          <t>Observability Completion: metrics everywhere</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr"/>
@@ -3587,7 +3644,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: error rate</t>
+          <t>Observability Completion: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr"/>
@@ -3603,7 +3660,7 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: requests/sec</t>
+          <t>Observability Completion: health checks everywhere</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr"/>
@@ -3619,7 +3676,7 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: DB connections</t>
+          <t>Observability Completion: dashboard: API latency</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr"/>
@@ -3635,7 +3692,7 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Kafka lag</t>
+          <t>Observability Completion: dashboard: error rate</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr"/>
@@ -3651,7 +3708,7 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: WebSocket connections</t>
+          <t>Observability Completion: dashboard: requests/sec</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr"/>
@@ -3667,7 +3724,7 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: Redis latency</t>
+          <t>Observability Completion: dashboard: DB connections</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr"/>
@@ -3683,7 +3740,7 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: notification failures</t>
+          <t>Observability Completion: dashboard: Kafka lag</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr"/>
@@ -3699,7 +3756,7 @@
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: dashboard: background job failures</t>
+          <t>Observability Completion: dashboard: WebSocket connections</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr"/>
@@ -3715,14 +3772,14 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Observability Completion: alerting rules</t>
+          <t>Observability Completion: dashboard: Redis latency</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B120" s="13" t="inlineStr">
         <is>
@@ -3731,14 +3788,14 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
+          <t>Observability Completion: dashboard: notification failures</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B121" s="13" t="inlineStr">
         <is>
@@ -3747,14 +3804,14 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
+          <t>Observability Completion: dashboard: background job failures</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B122" s="13" t="inlineStr">
         <is>
@@ -3763,7 +3820,7 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
+          <t>Observability Completion: alerting rules</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr"/>
@@ -3779,14 +3836,14 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
+          <t>Platform Control Plane: one view: applications/services/versions</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B124" s="13" t="inlineStr">
         <is>
@@ -3795,14 +3852,14 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
+          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B125" s="13" t="inlineStr">
         <is>
@@ -3811,14 +3868,14 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
+          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
@@ -3827,7 +3884,7 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
+          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr"/>
@@ -3843,7 +3900,7 @@
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
+          <t>AI Development Context: every module: README</t>
         </is>
       </c>
       <c r="D127" s="11" t="inlineStr"/>
@@ -3859,7 +3916,7 @@
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
+          <t>AI Development Context: every module: ownership metadata</t>
         </is>
       </c>
       <c r="D128" s="11" t="inlineStr"/>
@@ -3875,10 +3932,58 @@
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
+          <t>AI Development Context: every module: dependencies</t>
+        </is>
+      </c>
+      <c r="D129" s="11" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B130" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B131" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D131" s="11" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B132" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D129" s="11" t="inlineStr"/>
+      <c r="D132" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8592,7 +8697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9060,6 +9165,72 @@
       <c r="D21" s="11" t="inlineStr">
         <is>
           <t>Needs Node 20/22 and a real Yarn install - see platform/backstage/README.md if the versions on $PATH don't satisfy Backstage's own prerequisite check. Then open http://localhost:3000 (stop the Admin Portal first, they share a port) and browse the Catalog - every module/service/app is a real entity (Phase 26), not example fixture data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="48" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Test the Go SDK</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>cd packages/go/coresdk &amp;&amp; go test ./...</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>12 unit tests against a real httptest.Server (Phase 27) - no mocking library.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="48" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Test the TypeScript SDK</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>cd packages/typescript/core-sdk &amp;&amp; npm install &amp;&amp; npm test</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>13 unit tests against a real node:http server. make sdk-ts-build must run before apps/admin can resolve @core-platform/sdk - make admin-install/admin-build already depend on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="48" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Test the Dart SDK</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>cd packages/flutter/core_sdk &amp;&amp; dart pub get &amp;&amp; dart test</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>13 unit tests against a real dart:io HttpServer. apps/mobile depends on this package via a path: dependency in its pubspec.yaml.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 29
Roadmap/Todo/Stats/How-To-Test sheets updated for the control-plane
phase: Phase 29 marked Done with its real commit hash, Phase 30 (AI
Development Context) promoted to Next up, and a new How To Test step
for the /control-plane page. Also commits platform.json - Phase 29's
new machine-readable export that page reads, generated by this same
script from the same data as the xlsx workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -239,8 +239,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D135" headerRowCount="1">
-  <autoFilter ref="A1:D135"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D143" headerRowCount="1">
+  <autoFilter ref="A1:D143"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -281,8 +281,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D25" headerRowCount="1">
-  <autoFilter ref="A1:D25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="HowToTest" displayName="HowToTest" ref="A1:D26" headerRowCount="1">
+  <autoFilter ref="A1:D26"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Step"/>
     <tableColumn id="2" name="What"/>
@@ -633,12 +633,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>28 / 30</t>
+          <t>29 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>97%</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>apps/admin (Next.js 15 App Router)</t>
+          <t>apps/admin (Next.js 15 App Router) - now includes /control-plane, Phase 29</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>42</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1622,9 +1622,9 @@
       <c r="A30" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>One view of applications/services/versions/environments/dependencies/deployments/DB ownership/events/API contracts/health/alerts/recent changes - every module discoverable from one place.</t>
+          <t>New apps/admin/control-plane page - all 12 roadmap-named dimensions, real: applications/health (existing), real per-service versions (new config.Version - the actual git SHA, wired through health.Live/Health on all 3 services), real environment (from GET /v1/platform), the real dependency graph and DB ownership (docs/control/platform.json, a new machine-readable export from build_workbook.py's own data + catalog/system.yaml), real events (contracts/asyncapi), real live Prometheus alerts, a real git log for recent changes, and an honest Deployments placeholder (no CI/CD exists yet).</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>f0d1cc3</t>
         </is>
       </c>
     </row>
@@ -1647,9 +1647,9 @@
       <c r="A31" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Next up</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -1682,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2163,7 +2163,7 @@
     </row>
     <row r="30">
       <c r="A30" s="9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
@@ -2172,14 +2172,14 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+          <t>Phase 29: Platform Control Plane implemented, unit-tested, live-validated, documented, committed</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
@@ -2188,18 +2188,14 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
-        </is>
-      </c>
+          <t>Repo health baseline (make doctor / validate-all / go test / go build) run and passed</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="9" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
@@ -2208,32 +2204,32 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Separate Session table</t>
+          <t>Environment / ApplicationVersion / ApplicationConfiguration</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
+          <t>Deferred - no consumer needs them yet, documented as intentional in applications/README.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>5</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
+          <t>Separate Session table</t>
         </is>
       </c>
       <c r="D33" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
+          <t>Deferred - Device.SessionStatus covers today's single-session-per-device need, documented in devices/README.md</t>
         </is>
       </c>
     </row>
@@ -2248,12 +2244,12 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>UserPreferences (named in Phase 4, no fields ever specified)</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Known gap since Phase 9's audit, not yet picked up</t>
+          <t>Deferred to Phase 12+; notification preferences shipped, a generic preferences bag did not</t>
         </is>
       </c>
     </row>
@@ -2268,30 +2264,34 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>apps/admin next@15 / sharp transitive advisories</t>
+          <t>apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+          <t>Known gap since Phase 9's audit, not yet picked up</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>9</v>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Privacy: consent (append-only history)</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr"/>
+          <t>apps/admin next@15 / sharp transitive advisories</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Fix is a Next.js major-version bump - separate, reviewable change</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
+          <t>Privacy: consent (append-only history)</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr"/>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
+          <t>Privacy: user data export (ExportUserData registry - users/devices/files/audit)</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr"/>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
+          <t>Privacy: user deletion (DeleteUserData registry - users/devices/files; audit deliberately excluded)</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr"/>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Privacy: privacy preferences</t>
+          <t>Privacy: retention policy (declared, not scheduled - same documented gap as Phase 13's PurgeExpired)</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr"/>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+          <t>Privacy: privacy preferences</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr"/>
@@ -2377,21 +2377,17 @@
       <c r="A42" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B42" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Privacy: notifications module as an Export/Delete participant</t>
-        </is>
-      </c>
-      <c r="D42" s="11" t="inlineStr">
-        <is>
-          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
-        </is>
-      </c>
+          <t>Privacy: coordinate deletion through workflows/events - core-api's own embedded Temporal worker</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
@@ -2404,32 +2400,32 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>Privacy: relationships/groups/messaging as participants</t>
+          <t>Privacy: notifications module as an Export/Delete participant</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
+          <t>Deliberately deferred to prove the registry makes this a 2-line addition later, not a framework change</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="n">
-        <v>21</v>
-      </c>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>20</v>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Block</t>
+          <t>Privacy: relationships/groups/messaging as participants</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+          <t>Deferred - shared multi-user data needs a redaction strategy this phase's per-user-in-isolation registry doesn't fit</t>
         </is>
       </c>
     </row>
@@ -2444,10 +2440,14 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Mute</t>
-        </is>
-      </c>
-      <c r="D45" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: Block</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Reused Phase 8's relationships (Status='blocked'), deliberately not duplicated</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="n">
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
+          <t>Trust &amp; Safety: Mute</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr"/>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension</t>
+          <t>Trust &amp; Safety: Report -&gt; ModerationCase (deduplicated via partial unique index)</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr"/>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Ban</t>
+          <t>Trust &amp; Safety: Suspension</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr"/>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
+          <t>Trust &amp; Safety: Ban</t>
         </is>
       </c>
       <c r="D49" s="11" t="inlineStr"/>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
+          <t>Trust &amp; Safety: Appeal (approving lifts the target restriction)</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr"/>
@@ -2540,7 +2540,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
+          <t>Trust &amp; Safety: rate limiting (new platformkit/ratelimit, Valkey-backed)</t>
         </is>
       </c>
       <c r="D51" s="11" t="inlineStr"/>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
+          <t>Trust &amp; Safety: spam protection (5 reports/hour per reporter)</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr"/>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
+          <t>Trust &amp; Safety: abuse signals (critical severity auto-opens a case)</t>
         </is>
       </c>
       <c r="D53" s="11" t="inlineStr"/>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+          <t>Trust &amp; Safety: pluggable product-specific report reasons (free-form Reason field)</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr"/>
@@ -2597,21 +2597,17 @@
       <c r="A55" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
-        </is>
-      </c>
-      <c r="D55" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
-        </is>
-      </c>
+          <t>Trust &amp; Safety: Suspension/Ban actually restrict access (new requireActive middleware, one entry point)</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="9" t="n">
@@ -2624,30 +2620,34 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+          <t>Trust &amp; Safety: WebSocket disconnect on suspension/ban</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+          <t>Deferred - only HTTP access is gated; an existing realtime-gateway connection isn't forcibly closed</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>22</v>
-      </c>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>21</v>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Billing: Payment model (provider-specific transaction record)</t>
-        </is>
-      </c>
-      <c r="D57" s="11" t="inlineStr"/>
+          <t>Trust &amp; Safety: aggregating lower-severity signals over a time window</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - a real abuse-detection engine is out of this phase's scope; only single-critical-signal escalation is implemented</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="n">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
+          <t>Billing: Payment model (provider-specific transaction record)</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+          <t>Billing: Entitlement model (platform-facing truth, kept separate from Payment)</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr"/>
@@ -2692,32 +2692,28 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Billing: Stripe adapter</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
-        </is>
-      </c>
+          <t>Billing: provider abstraction (PaymentProvider interface + registry, implemented first)</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Billing: Apple IAP adapter</t>
+          <t>Billing: Stripe adapter</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
+          <t>Real HMAC-SHA256 webhook signature verification, live-validated without a Stripe account via self-signed test payloads</t>
         </is>
       </c>
     </row>
@@ -2732,30 +2728,34 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Billing: Google Play adapter</t>
+          <t>Billing: Apple IAP adapter</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+          <t>Deferred - needs real App Store Server API credentials this environment doesn't have</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
-        <v>23</v>
-      </c>
-      <c r="B63" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>22</v>
+      </c>
+      <c r="B63" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
-        </is>
-      </c>
-      <c r="D63" s="11" t="inlineStr"/>
+          <t>Billing: Google Play adapter</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - needs real Play Developer API credentials this environment doesn't have</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
+          <t>Analytics: generic event envelope (event_name/user_id/anonymous_id/app_id/session_id/timestamp/properties/context)</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr"/>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+          <t>Analytics: keep operational DBs out of the analytics path (analytics_events is a landing buffer, never queried for analytics)</t>
         </is>
       </c>
       <c r="D65" s="11" t="inlineStr"/>
@@ -2793,37 +2793,37 @@
       <c r="A66" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B66" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
-        </is>
-      </c>
-      <c r="D66" s="11" t="inlineStr">
-        <is>
-          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
-        </is>
-      </c>
+          <t>Analytics: pipeline foundation for ClickHouse/warehouse/data lake (worker batches NDJSON into MinIO/S3)</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="B67" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>23</v>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
-        </is>
-      </c>
-      <c r="D67" s="11" t="inlineStr"/>
+          <t>Analytics: an actual ClickHouse/warehouse/data-lake query layer</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>Out of scope - this phase builds the landing pipeline only; no real destination system exists in this environment to integrate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
@@ -2836,32 +2836,28 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: local models / Ollama adapter</t>
-        </is>
-      </c>
-      <c r="D68" s="11" t="inlineStr">
-        <is>
-          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
-        </is>
-      </c>
+          <t>AI Gateway: provider-neutral interface (Provider: Name + Complete)</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B69" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: OpenAI adapter</t>
+          <t>AI Gateway: local models / Ollama adapter</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no real API key in this environment to validate against honestly</t>
+          <t>Real local inference via a new Ollama container, auto-pulled model, no vendor API key - the one live-testable provider</t>
         </is>
       </c>
     </row>
@@ -2876,7 +2872,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Anthropic adapter</t>
+          <t>AI Gateway: OpenAI adapter</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
@@ -2896,7 +2892,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: Google adapter</t>
+          <t>AI Gateway: Anthropic adapter</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
@@ -2909,17 +2905,21 @@
       <c r="A72" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B72" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
-        </is>
-      </c>
-      <c r="D72" s="11" t="inlineStr"/>
+          <t>AI Gateway: Google adapter</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - no real API key in this environment to validate against honestly</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="n">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
+          <t>AI Gateway: model routing (product-facing ModelAlias, never a vendor model name)</t>
         </is>
       </c>
       <c r="D73" s="11" t="inlineStr"/>
@@ -2948,7 +2948,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: token usage tracking</t>
+          <t>AI Gateway: quotas (ratelimit.Limiter reused a third time, 60/min/caller)</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr"/>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
+          <t>AI Gateway: token usage tracking</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr"/>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="C76" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
+          <t>AI Gateway: cost tracking (real per-route price table; Ollama honestly priced at 0)</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr"/>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
+          <t>AI Gateway: audit integration (new AIGatewayAuditRecorder, a genuine audit.Record per call)</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr"/>
@@ -3012,7 +3012,7 @@
       </c>
       <c r="C78" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
+          <t>AI Gateway: prompt/version metadata (free-form PromptKey/PromptVersion)</t>
         </is>
       </c>
       <c r="D78" s="11" t="inlineStr"/>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+          <t>AI Gateway: timeouts (context.WithTimeout per provider call)</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr"/>
@@ -3037,37 +3037,37 @@
       <c r="A80" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B80" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
-        </is>
-      </c>
-      <c r="D80" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
-        </is>
-      </c>
+          <t>AI Gateway: fallback (ordered provider/model chain, first success wins)</t>
+        </is>
+      </c>
+      <c r="D80" s="11" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="B81" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>24</v>
+      </c>
+      <c r="B81" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
-        </is>
-      </c>
-      <c r="D81" s="11" t="inlineStr"/>
+          <t>AI Gateway: live token-quantity quota (as opposed to today's call-count quota)</t>
+        </is>
+      </c>
+      <c r="D81" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - Repository already has the data (Completion.TotalTokens); not wired as a live gate yet</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="n">
@@ -3080,14 +3080,10 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Applications</t>
-        </is>
-      </c>
-      <c r="D82" s="11" t="inlineStr">
-        <is>
-          <t>Real GET /v1/apps table</t>
-        </is>
-      </c>
+          <t>Admin Portal: real Keycloak-authenticated session (Resource Owner Password Credentials grant), httpOnly session cookie</t>
+        </is>
+      </c>
+      <c r="D82" s="11" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="9" t="n">
@@ -3100,12 +3096,12 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Users (list + detail)</t>
+          <t>Admin Portal: visibility - Applications</t>
         </is>
       </c>
       <c r="D83" s="11" t="inlineStr">
         <is>
-          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
+          <t>Real GET /v1/apps table</t>
         </is>
       </c>
     </row>
@@ -3120,12 +3116,12 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Roles/Permissions</t>
+          <t>Admin Portal: visibility - Users (list + detail)</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+          <t>New admin-wide GET /v1/users (cursor-paginated, platform.admin-gated)</t>
         </is>
       </c>
     </row>
@@ -3140,10 +3136,14 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
-        </is>
-      </c>
-      <c r="D85" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - Roles/Permissions</t>
+        </is>
+      </c>
+      <c r="D85" s="11" t="inlineStr">
+        <is>
+          <t>New authz HTTP surface (GET/POST /v1/authz/roles, POST /v1/authz/roles/revoke) with a full grant/revoke UI</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="n">
@@ -3156,7 +3156,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Moderation, Audit</t>
+          <t>Admin Portal: visibility - Feature Flags, Configuration, Jobs</t>
         </is>
       </c>
       <c r="D86" s="11" t="inlineStr"/>
@@ -3172,14 +3172,10 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - System Health</t>
-        </is>
-      </c>
-      <c r="D87" s="11" t="inlineStr">
-        <is>
-          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Moderation, Audit</t>
+        </is>
+      </c>
+      <c r="D87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="9" t="n">
@@ -3192,30 +3188,30 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
-        </is>
-      </c>
-      <c r="D88" s="11" t="inlineStr"/>
+          <t>Admin Portal: visibility - System Health</t>
+        </is>
+      </c>
+      <c r="D88" s="11" t="inlineStr">
+        <is>
+          <t>Live GET /healthz against core-api/realtime-gateway/worker</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B89" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B89" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
-        </is>
-      </c>
-      <c r="D89" s="11" t="inlineStr">
-        <is>
-          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
-        </is>
-      </c>
+          <t>Admin Portal: visibility - Billing, AI Gateway usage (bonus, not roadmap-named)</t>
+        </is>
+      </c>
+      <c r="D89" s="11" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="9" t="n">
@@ -3228,32 +3224,32 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Admin Portal: visibility - Deployments</t>
+          <t>Admin Portal: visibility - Sessions/Devices, Tenants, Relationships, Messages, Notifications, Files</t>
         </is>
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
+          <t>Deferred - each backing module only exposes a listMine-style self-scoped endpoint, not an admin-wide one; honest ComingSoon reasoning shown per area instead of fake rows</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="B91" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>25</v>
+      </c>
+      <c r="B91" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Backstage: integrate Backstage as developer portal</t>
+          <t>Admin Portal: visibility - Deployments</t>
         </is>
       </c>
       <c r="D91" s="11" t="inlineStr">
         <is>
-          <t>Real @backstage/create-app instance at platform/backstage, catalog wired to real catalog/*.yaml + contracts/*/catalog-info.yaml, live-validated via the real catalog API (21 Components, 2 APIs, 1 System, 1 Group, 0 processing errors)</t>
+          <t>Deferred to Phase 29 - nothing in the platform tracks deployments as data yet</t>
         </is>
       </c>
     </row>
@@ -3268,12 +3264,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - name/description/owner/lifecycle</t>
+          <t>Backstage: integrate Backstage as developer portal</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>All 16 modules/*/module.yaml + README.md real (11 were still stub text before this phase)</t>
+          <t>Real @backstage/create-app instance at platform/backstage, catalog wired to real catalog/*.yaml + contracts/*/catalog-info.yaml, live-validated via the real catalog API (21 Components, 2 APIs, 1 System, 1 Group, 0 processing errors)</t>
         </is>
       </c>
     </row>
@@ -3288,12 +3284,12 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - repository/documentation</t>
+          <t>Backstage: per-module metadata - name/description/owner/lifecycle</t>
         </is>
       </c>
       <c r="D93" s="11" t="inlineStr">
         <is>
-          <t>Every Component links its module README; the System entity links VALIDATION.md and the new docs/RUNBOOKS.md</t>
+          <t>All 16 modules/*/module.yaml + README.md real (11 were still stub text before this phase)</t>
         </is>
       </c>
     </row>
@@ -3308,12 +3304,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - dependencies</t>
+          <t>Backstage: per-module metadata - repository/documentation</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Component dependsOn mirrors modules/*/module.yaml's real dependency graph; Backstage computes reverse dependencyOf relations automatically, confirmed live</t>
+          <t>Every Component links its module README; the System entity links VALIDATION.md and the new docs/RUNBOOKS.md</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3324,12 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - APIs</t>
+          <t>Backstage: per-module metadata - dependencies</t>
         </is>
       </c>
       <c r="D95" s="11" t="inlineStr">
         <is>
-          <t>2 API entities (OpenAPI, AsyncAPI), both with their full real spec embedded and live-loaded</t>
+          <t>Component dependsOn mirrors modules/*/module.yaml's real dependency graph; Backstage computes reverse dependencyOf relations automatically, confirmed live</t>
         </is>
       </c>
     </row>
@@ -3348,12 +3344,12 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - events</t>
+          <t>Backstage: per-module metadata - APIs</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>providesApis set only on the components whose code actually calls outbox.Record, cross-checked against the real Go source</t>
+          <t>2 API entities (OpenAPI, AsyncAPI), both with their full real spec embedded and live-loaded</t>
         </is>
       </c>
     </row>
@@ -3361,19 +3357,19 @@
       <c r="A97" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B97" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B97" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - database ownership</t>
+          <t>Backstage: per-module metadata - events</t>
         </is>
       </c>
       <c r="D97" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no per-module DB-ownership annotation convention chosen yet; docs/control's Modules sheet tracks this today at a finer grain than catalog/system.yaml's 16 domains</t>
+          <t>providesApis set only on the components whose code actually calls outbox.Record, cross-checked against the real Go source</t>
         </is>
       </c>
     </row>
@@ -3381,19 +3377,19 @@
       <c r="A98" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B98" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B98" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - dashboards</t>
+          <t>Backstage: per-module metadata - database ownership</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>core-platform.io/dashboard annotation on each service pointing at the real local Grafana instance - no per-service dashboard exists yet (that's Phase 28), so it points at the shared instance, documented as such</t>
+          <t>Deferred - no per-module DB-ownership annotation convention chosen yet; docs/control's Modules sheet tracks this today at a finer grain than catalog/system.yaml's 16 domains</t>
         </is>
       </c>
     </row>
@@ -3408,18 +3404,18 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Backstage: per-module metadata - runbooks</t>
+          <t>Backstage: per-module metadata - dashboards</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>New docs/RUNBOOKS.md, linked from the System entity</t>
+          <t>core-platform.io/dashboard annotation on each service pointing at the real local Grafana instance - no per-service dashboard exists yet (that's Phase 28), so it points at the shared instance, documented as such</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
@@ -3428,12 +3424,12 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Go SDK</t>
+          <t>Backstage: per-module metadata - runbooks</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>packages/go/coresdk - 12 unit tests (httptest.Server), live-validated against real Keycloak/core-api/realtime-gateway</t>
+          <t>New docs/RUNBOOKS.md, linked from the System entity</t>
         </is>
       </c>
     </row>
@@ -3448,12 +3444,12 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>SDKs: TypeScript SDK</t>
+          <t>SDKs: Go SDK</t>
         </is>
       </c>
       <c r="D101" s="11" t="inlineStr">
         <is>
-          <t>packages/typescript/core-sdk - 13 unit tests (node:http), real consumer: apps/admin's entire lib/api.ts migrated to it</t>
+          <t>packages/go/coresdk - 12 unit tests (httptest.Server), live-validated against real Keycloak/core-api/realtime-gateway</t>
         </is>
       </c>
     </row>
@@ -3468,12 +3464,12 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>SDKs: Dart SDK</t>
+          <t>SDKs: TypeScript SDK</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>packages/flutter/core_sdk (pure Dart, no Flutter dependency) - 13 unit tests (dart:io HttpServer), real consumer: apps/mobile's login/profile flow</t>
+          <t>packages/typescript/core-sdk - 13 unit tests (node:http), real consumer: apps/admin's entire lib/api.ts migrated to it</t>
         </is>
       </c>
     </row>
@@ -3488,12 +3484,12 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>SDKs: auth + token refresh in each SDK</t>
+          <t>SDKs: Dart SDK</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>TokenSource (static + real Keycloak password-grant with skew-aware, concurrency-coalesced refresh) in all three</t>
+          <t>packages/flutter/core_sdk (pure Dart, no Flutter dependency) - 13 unit tests (dart:io HttpServer), real consumer: apps/mobile's login/profile flow</t>
         </is>
       </c>
     </row>
@@ -3508,12 +3504,12 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>SDKs: pagination + safe retries</t>
+          <t>SDKs: auth + token refresh in each SDK</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>Page/paginate/collectAll over the real {items,nextCursor} shape; GET-only retries by default on transient statuses, in all three</t>
+          <t>TokenSource (static + real Keycloak password-grant with skew-aware, concurrency-coalesced refresh) in all three</t>
         </is>
       </c>
     </row>
@@ -3528,12 +3524,12 @@
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>SDKs: realtime connection helper</t>
+          <t>SDKs: pagination + safe retries</t>
         </is>
       </c>
       <c r="D105" s="11" t="inlineStr">
         <is>
-          <t>Reproduces realtime-gateway's real ws://.../ws?access_token=&amp;deviceId= protocol and message shapes exactly, in all three - live-validated with real cross-connection fan-out</t>
+          <t>Page/paginate/collectAll over the real {items,nextCursor} shape; GET-only retries by default on transient statuses, in all three</t>
         </is>
       </c>
     </row>
@@ -3548,12 +3544,12 @@
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>SDKs: correlation ID propagation</t>
+          <t>SDKs: realtime connection helper</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>X-Correlation-ID on every call, matching platformkit/correlation's real header name, in all three</t>
+          <t>Reproduces realtime-gateway's real ws://.../ws?access_token=&amp;deviceId= protocol and message shapes exactly, in all three - live-validated with real cross-connection fan-out</t>
         </is>
       </c>
     </row>
@@ -3568,12 +3564,12 @@
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>SDKs: device registration helper</t>
+          <t>SDKs: correlation ID propagation</t>
         </is>
       </c>
       <c r="D107" s="11" t="inlineStr">
         <is>
-          <t>DevicesRegister/devicesRegister in all three - realtime dial requires a real registered device id</t>
+          <t>X-Correlation-ID on every call, matching platformkit/correlation's real header name, in all three</t>
         </is>
       </c>
     </row>
@@ -3588,12 +3584,12 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>SDKs: apps/mobile test/ directory (make flutter-test currently fails)</t>
+          <t>SDKs: device registration helper</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>Closed as a side effect - real widget tests added, discovered and worked around Flutter's TestWidgetsFlutterBinding network-mocking constraint live. Was pending since Phase 9.</t>
+          <t>DevicesRegister/devicesRegister in all three - realtime dial requires a real registered device id</t>
         </is>
       </c>
     </row>
@@ -3601,39 +3597,39 @@
       <c r="A109" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B109" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B109" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>SDKs: full API coverage (all 146 endpoints typed) in each SDK</t>
+          <t>SDKs: apps/mobile test/ directory (make flutter-test currently fails)</t>
         </is>
       </c>
       <c r="D109" s="11" t="inlineStr">
         <is>
-          <t>Deferred - each SDK covers a representative 'core identity' slice (platform/identity/users/devices/applications) plus what its real consumer needs; the untyped request()/Do() escape hatch reaches everything else. Broader coverage is real, additive work, not a framework limitation.</t>
+          <t>Closed as a side effect - real widget tests added, discovered and worked around Flutter's TestWidgetsFlutterBinding network-mocking constraint live. Was pending since Phase 9.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B110" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+        <v>27</v>
+      </c>
+      <c r="B110" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Observability: structured logs everywhere</t>
+          <t>SDKs: full API coverage (all 146 endpoints typed) in each SDK</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>logging.NewWithLoki ships every record to Loki's real push API directly; on by default locally (LOKI_PUSH_URL)</t>
+          <t>Deferred - each SDK covers a representative 'core identity' slice (platform/identity/users/devices/applications) plus what its real consumer needs; the untyped request()/Do() escape hatch reaches everything else. Broader coverage is real, additive work, not a framework limitation.</t>
         </is>
       </c>
     </row>
@@ -3648,12 +3644,12 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Observability: metrics everywhere</t>
+          <t>Observability: structured logs everywhere</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>New packages/go/platformkit/metrics - real GET /metrics (Prometheus exposition) on core-api, realtime-gateway, and worker</t>
+          <t>logging.NewWithLoki ships every record to Loki's real push API directly; on by default locally (LOKI_PUSH_URL)</t>
         </is>
       </c>
     </row>
@@ -3668,12 +3664,12 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Observability: distributed traces everywhere</t>
+          <t>Observability: metrics everywhere</t>
         </is>
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>Already real since Phase 1 (otelx) - confirmed still working live this phase</t>
+          <t>New packages/go/platformkit/metrics - real GET /metrics (Prometheus exposition) on core-api, realtime-gateway, and worker</t>
         </is>
       </c>
     </row>
@@ -3688,12 +3684,12 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Observability: health checks everywhere</t>
+          <t>Observability: distributed traces everywhere</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>Already real since Phase 1 (/livez /readyz /healthz) - confirmed still working live this phase</t>
+          <t>Already real since Phase 1 (otelx) - confirmed still working live this phase</t>
         </is>
       </c>
     </row>
@@ -3708,12 +3704,12 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - API latency</t>
+          <t>Observability: health checks everywhere</t>
         </is>
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>http_request_duration_seconds, labeled by route pattern (not raw path) to keep cardinality bounded</t>
+          <t>Already real since Phase 1 (/livez /readyz /healthz) - confirmed still working live this phase</t>
         </is>
       </c>
     </row>
@@ -3728,12 +3724,12 @@
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - error rate</t>
+          <t>Observability: dashboard - API latency</t>
         </is>
       </c>
       <c r="D115" s="11" t="inlineStr">
         <is>
-          <t>http_requests_total{status=~"5.."} / http_requests_total</t>
+          <t>http_request_duration_seconds, labeled by route pattern (not raw path) to keep cardinality bounded</t>
         </is>
       </c>
     </row>
@@ -3748,12 +3744,12 @@
       </c>
       <c r="C116" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - requests/sec</t>
+          <t>Observability: dashboard - error rate</t>
         </is>
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>rate(http_requests_total[5m])</t>
+          <t>http_requests_total{status=~"5.."} / http_requests_total</t>
         </is>
       </c>
     </row>
@@ -3768,12 +3764,12 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - DB connections</t>
+          <t>Observability: dashboard - requests/sec</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>db_pool_connections, real pgxpool.Stat() polled on a ticker (pg.ReportStats) on all 3 services</t>
+          <t>rate(http_requests_total[5m])</t>
         </is>
       </c>
     </row>
@@ -3781,19 +3777,19 @@
       <c r="A118" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B118" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B118" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C118" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - Kafka lag</t>
+          <t>Observability: dashboard - DB connections</t>
         </is>
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>Deliberately not implemented - no real Kafka/Redpanda producer or consumer exists in this codebase yet (documented since Phase 14); an honest placeholder panel explains this instead of a fabricated metric</t>
+          <t>db_pool_connections, real pgxpool.Stat() polled on a ticker (pg.ReportStats) on all 3 services</t>
         </is>
       </c>
     </row>
@@ -3801,19 +3797,19 @@
       <c r="A119" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B119" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="B119" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - WebSocket connections</t>
+          <t>Observability: dashboard - Kafka lag</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>realtime_ws_connections, live-validated going 0 -&gt; 1 -&gt; 0 across a real connect/hold/disconnect cycle against the running service</t>
+          <t>Deliberately not implemented - no real Kafka/Redpanda producer or consumer exists in this codebase yet (documented since Phase 14); an honest placeholder panel explains this instead of a fabricated metric</t>
         </is>
       </c>
     </row>
@@ -3828,12 +3824,12 @@
       </c>
       <c r="C120" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - Redis latency</t>
+          <t>Observability: dashboard - WebSocket connections</t>
         </is>
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>redis_command_duration_seconds via a real go-redis v9 Hook, InstrumentRedis</t>
+          <t>realtime_ws_connections, live-validated going 0 -&gt; 1 -&gt; 0 across a real connect/hold/disconnect cycle against the running service</t>
         </is>
       </c>
     </row>
@@ -3848,12 +3844,12 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - notification failures</t>
+          <t>Observability: dashboard - Redis latency</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>notification_delivery_failures_total, incremented at notifications.Service.dispatch's two real failure paths</t>
+          <t>redis_command_duration_seconds via a real go-redis v9 Hook, InstrumentRedis</t>
         </is>
       </c>
     </row>
@@ -3868,12 +3864,12 @@
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>Observability: dashboard - background job failures</t>
+          <t>Observability: dashboard - notification failures</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>job_failures_total, incremented only on jobrunner's real dead_letter transition (not every retryable attempt)</t>
+          <t>notification_delivery_failures_total, incremented at notifications.Service.dispatch's two real failure paths</t>
         </is>
       </c>
     </row>
@@ -3888,12 +3884,12 @@
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>Observability: alerting rules</t>
+          <t>Observability: dashboard - background job failures</t>
         </is>
       </c>
       <c r="D123" s="11" t="inlineStr">
         <is>
-          <t>6 real, live-evaluated Prometheus rules (infra/observability/alerts.yml) - ServiceDown live-confirmed firing then clearing on the real service lifecycle</t>
+          <t>job_failures_total, incremented only on jobrunner's real dead_letter transition (not every retryable attempt)</t>
         </is>
       </c>
     </row>
@@ -3901,19 +3897,19 @@
       <c r="A124" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B124" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B124" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Observability: Alertmanager routing (Slack/PagerDuty/email)</t>
+          <t>Observability: alerting rules</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>Deferred - no real notification-channel credentials in this environment, the same reasoning Stripe/AI vendor adapters have documented; Prometheus's own rule evaluation and API are real regardless</t>
+          <t>6 real, live-evaluated Prometheus rules (infra/observability/alerts.yml) - ServiceDown live-confirmed firing then clearing on the real service lifecycle</t>
         </is>
       </c>
     </row>
@@ -3928,18 +3924,18 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Observability: per-service (not shared) Grafana dashboards</t>
+          <t>Observability: Alertmanager routing (Slack/PagerDuty/email)</t>
         </is>
       </c>
       <c r="D125" s="11" t="inlineStr">
         <is>
-          <t>Deferred - one shared 'Core Platform Overview' dashboard covers all 3 services today, not 9 separate roadmap-named dashboards</t>
+          <t>Deferred - no real notification-channel credentials in this environment, the same reasoning Stripe/AI vendor adapters have documented; Prometheus's own rule evaluation and API are real regardless</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B126" s="13" t="inlineStr">
         <is>
@@ -3948,78 +3944,98 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: applications/services/versions</t>
-        </is>
-      </c>
-      <c r="D126" s="11" t="inlineStr"/>
+          <t>Observability: per-service (not shared) Grafana dashboards</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>Deferred - one shared 'Core Platform Overview' dashboard covers all 3 services today, not 9 separate roadmap-named dashboards</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B127" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B127" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C127" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: environments/dependencies/deployments</t>
-        </is>
-      </c>
-      <c r="D127" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - applications/services</t>
+        </is>
+      </c>
+      <c r="D127" s="11" t="inlineStr">
+        <is>
+          <t>New apps/admin/control-plane page, real GET /v1/apps + per-service health</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B128" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C128" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: DB ownership/events/API contracts</t>
-        </is>
-      </c>
-      <c r="D128" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - versions</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>New config.Version (real git SHA via `git rev-parse --short HEAD`, BUILD_VERSION override) wired through health.Live/Health on all 3 services</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B129" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B129" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C129" s="11" t="inlineStr">
         <is>
-          <t>Platform Control Plane: one view: health/alerts/recent changes</t>
-        </is>
-      </c>
-      <c r="D129" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - environments</t>
+        </is>
+      </c>
+      <c r="D129" s="11" t="inlineStr">
+        <is>
+          <t>Read live from GET /v1/platform's environment field - one real entry, not a fabricated multi-env list</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B130" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>29</v>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C130" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
-        </is>
-      </c>
-      <c r="D130" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - dependencies</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>New docs/control/platform.json (build_workbook.py export) parses catalog/system.yaml's real dependsOn graph - 23 components</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="9" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B131" s="13" t="inlineStr">
         <is>
@@ -4028,74 +4044,230 @@
       </c>
       <c r="C131" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
-        </is>
-      </c>
-      <c r="D131" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - deployments</t>
+        </is>
+      </c>
+      <c r="D131" s="11" t="inlineStr">
+        <is>
+          <t>Honest placeholder - no CI/CD pipeline or deployment tracking exists in this environment; real per-service version is the closest honest signal today</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B132" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>29</v>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C132" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
-        </is>
-      </c>
-      <c r="D132" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - DB ownership</t>
+        </is>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>platform.json exports the same module/storage data docs/control's Modules sheet tracks - one source, not a third copy</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B133" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>29</v>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C133" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
-        </is>
-      </c>
-      <c r="D133" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - events</t>
+        </is>
+      </c>
+      <c r="D133" s="11" t="inlineStr">
+        <is>
+          <t>platform.json parses contracts/asyncapi/events.yaml's real channels</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="B134" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+        <v>29</v>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
-        </is>
-      </c>
-      <c r="D134" s="11" t="inlineStr"/>
+          <t>Control Plane: one view - API contracts</t>
+        </is>
+      </c>
+      <c r="D134" s="11" t="inlineStr">
+        <is>
+          <t>Links to the real OpenAPI/AsyncAPI files and the Backstage catalog (Phase 26)</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B135" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C135" s="11" t="inlineStr">
+        <is>
+          <t>Control Plane: one view - health</t>
+        </is>
+      </c>
+      <c r="D135" s="11" t="inlineStr">
+        <is>
+          <t>Reuses the existing real getSystemHealth() live /healthz calls</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C136" s="11" t="inlineStr">
+        <is>
+          <t>Control Plane: one view - alerts</t>
+        </is>
+      </c>
+      <c r="D136" s="11" t="inlineStr">
+        <is>
+          <t>New live fetch of Prometheus's real GET /api/v1/alerts (Phase 28's rules) - cross-checked live against a direct curl to the same endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="B137" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C137" s="11" t="inlineStr">
+        <is>
+          <t>Control Plane: one view - recent changes</t>
+        </is>
+      </c>
+      <c r="D137" s="11" t="inlineStr">
+        <is>
+          <t>New real `git log` of the checkout, run server-side - not a hand-maintained changelog</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B135" s="13" t="inlineStr">
+      <c r="B138" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="C135" s="11" t="inlineStr">
+      <c r="C138" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: README</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B139" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C139" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: ownership metadata</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B140" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C140" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: dependencies</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B141" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C141" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: API contract</t>
+        </is>
+      </c>
+      <c r="D141" s="11" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B142" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C142" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module: event contracts</t>
+        </is>
+      </c>
+      <c r="D142" s="11" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B143" s="13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C143" s="11" t="inlineStr">
         <is>
           <t>AI Development Context: every module: DB ownership</t>
         </is>
       </c>
-      <c r="D135" s="11" t="inlineStr"/>
+      <c r="D143" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8836,7 +9008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9392,6 +9564,28 @@
       <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Needs core-api/realtime-gateway/worker actually running (steps 5-7). Every panel is real data (Phase 28) - API latency, error rate, requests/sec, DB connections, WebSocket connections, Redis latency, notification/job failures. Prometheus alerts: http://localhost:9090/alerts. Loki/Tempo: query via Grafana's Explore tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="48" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>See the whole platform in one view</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Sign into the Admin Portal (step 19), then Overview -&gt; Control Plane</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Phase 29 - applications, per-service health/real versions (git SHA), environment, the real dependency graph, database ownership, events, API contract links, live Prometheus alerts, and a real git log, all on one real page. Prometheus (step 24's stack) must be running for the Alerts section to show live data - it degrades to an honest empty list otherwise, not an error.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(control): update dashboard through Phase 30
Roadmap complete: 30/30 phases (100%). Marks Phase 30 Done in the
roadmap and todo checklist, regenerates data.xlsx/index.html/
platform.json from the same generation script so the dashboard,
Backstage catalog data, and Admin Portal control-plane page cannot
drift apart.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/control/data.xlsx
+++ b/docs/control/data.xlsx
@@ -63,7 +63,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -78,11 +78,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -117,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,9 +138,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -239,8 +231,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D143" headerRowCount="1">
-  <autoFilter ref="A1:D143"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TodoChecklist" displayName="TodoChecklist" ref="A1:D146" headerRowCount="1">
+  <autoFilter ref="A1:D146"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Phase"/>
     <tableColumn id="2" name="Status"/>
@@ -633,12 +625,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>29 / 30</t>
+          <t>30 / 30</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -803,7 +795,7 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1647,9 +1639,9 @@
       <c r="A31" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Next up</t>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -1659,7 +1651,7 @@
       </c>
       <c r="D31" s="11" t="inlineStr">
         <is>
-          <t>Machine-readable context for AI agents - every module carries README, ownership metadata, dependencies, API contract, event contracts, DB ownership, so an agent (like this one) can safely work on any part of the platform.</t>
+          <t>Audited and confirmed real per-module README/ownership/dependencies/API+event contracts/DB ownership already existed (Phases 26/29); closed the one genuine gap - 12 of 22 core-api modules had no handler-level (http_test.go) coverage - with real tests reading each module's actual source, never assumed. Rewrote docs/AI_CONTEXT.md and docs/architecture/overview.md from stale initial-commit stubs into a real description of the module pattern, testing convention, real-infra-only validation philosophy, and the phase loop this whole build actually followed.</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
@@ -1682,7 +1674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D143"/>
+  <dimension ref="A1:D146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2237,7 +2229,7 @@
       <c r="A34" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2257,7 +2249,7 @@
       <c r="A35" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2277,7 +2269,7 @@
       <c r="A36" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2393,7 +2385,7 @@
       <c r="A43" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B43" s="13" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2413,7 +2405,7 @@
       <c r="A44" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="B44" s="13" t="inlineStr">
+      <c r="B44" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2613,7 +2605,7 @@
       <c r="A56" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B56" s="13" t="inlineStr">
+      <c r="B56" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2633,7 +2625,7 @@
       <c r="A57" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="B57" s="13" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2721,7 +2713,7 @@
       <c r="A62" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B62" s="13" t="inlineStr">
+      <c r="B62" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2741,7 +2733,7 @@
       <c r="A63" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="B63" s="13" t="inlineStr">
+      <c r="B63" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2809,7 +2801,7 @@
       <c r="A67" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="B67" s="13" t="inlineStr">
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2865,7 +2857,7 @@
       <c r="A70" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B70" s="13" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2885,7 +2877,7 @@
       <c r="A71" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B71" s="13" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -2905,7 +2897,7 @@
       <c r="A72" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B72" s="13" t="inlineStr">
+      <c r="B72" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3053,7 +3045,7 @@
       <c r="A81" s="9" t="n">
         <v>24</v>
       </c>
-      <c r="B81" s="13" t="inlineStr">
+      <c r="B81" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3217,7 +3209,7 @@
       <c r="A90" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B90" s="13" t="inlineStr">
+      <c r="B90" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3237,7 +3229,7 @@
       <c r="A91" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="B91" s="13" t="inlineStr">
+      <c r="B91" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3377,7 +3369,7 @@
       <c r="A98" s="9" t="n">
         <v>26</v>
       </c>
-      <c r="B98" s="13" t="inlineStr">
+      <c r="B98" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3617,7 +3609,7 @@
       <c r="A110" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="B110" s="13" t="inlineStr">
+      <c r="B110" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3797,7 +3789,7 @@
       <c r="A119" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B119" s="13" t="inlineStr">
+      <c r="B119" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3917,7 +3909,7 @@
       <c r="A125" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B125" s="13" t="inlineStr">
+      <c r="B125" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -3937,7 +3929,7 @@
       <c r="A126" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="B126" s="13" t="inlineStr">
+      <c r="B126" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -4037,7 +4029,7 @@
       <c r="A131" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="B131" s="13" t="inlineStr">
+      <c r="B131" s="12" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -4177,97 +4169,181 @@
       <c r="A138" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B138" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C138" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: README</t>
-        </is>
-      </c>
-      <c r="D138" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - README</t>
+        </is>
+      </c>
+      <c r="D138" s="11" t="inlineStr">
+        <is>
+          <t>backend/core-api/internal/&lt;module&gt;/README.md - real Responsibilities/Non-responsibilities/Layout/Storage sections, the actual architecture notes (already real since early phases, confirmed this phase)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B139" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C139" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: ownership metadata</t>
-        </is>
-      </c>
-      <c r="D139" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - ownership metadata</t>
+        </is>
+      </c>
+      <c r="D139" s="11" t="inlineStr">
+        <is>
+          <t>modules/*/module.yaml (owner/lifecycle) - real since Phase 26</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B140" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C140" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: dependencies</t>
-        </is>
-      </c>
-      <c r="D140" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - dependencies</t>
+        </is>
+      </c>
+      <c r="D140" s="11" t="inlineStr">
+        <is>
+          <t>modules/*/module.yaml + catalog/system.yaml's dependsOn graph - real since Phase 26</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B141" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C141" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: API contract</t>
-        </is>
-      </c>
-      <c r="D141" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - API contract</t>
+        </is>
+      </c>
+      <c r="D141" s="11" t="inlineStr">
+        <is>
+          <t>contracts/openapi/core-api.yaml, module-prefixed operationIds - real since Phase 26</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B142" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C142" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: event contracts</t>
-        </is>
-      </c>
-      <c r="D142" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - event contracts</t>
+        </is>
+      </c>
+      <c r="D142" s="11" t="inlineStr">
+        <is>
+          <t>contracts/asyncapi/events.yaml, cross-checked against real outbox.Record call sites - real since Phase 26</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B143" s="13" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="C143" s="11" t="inlineStr">
         <is>
-          <t>AI Development Context: every module: DB ownership</t>
-        </is>
-      </c>
-      <c r="D143" s="11" t="inlineStr"/>
+          <t>AI Development Context: every module - DB ownership</t>
+        </is>
+      </c>
+      <c r="D143" s="11" t="inlineStr">
+        <is>
+          <t>docs/control/platform.json's Modules export - real since Phase 29</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C144" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: every module - tests</t>
+        </is>
+      </c>
+      <c r="D144" s="11" t="inlineStr">
+        <is>
+          <t>Service-layer tests were already real everywhere; closed the real gap this phase found - 12 of 22 core-api modules (aigateway, analytics, audit, authz, billing, features, jobs, privacy, remoteconfig, search, trustsafety, workflows) had no http_test.go handler-layer coverage. All 12 now have 3-5 tests each against the real router, reading actual source rather than assumed shapes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C145" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: docs/AI_CONTEXT.md reflects real architecture rules</t>
+        </is>
+      </c>
+      <c r="D145" s="11" t="inlineStr">
+        <is>
+          <t>Rewritten from a 26-line initial-commit stub into a real description of the layered module pattern, consumer-defined interfaces, two-phase wiring, the testing convention, real-infra-only validation, the catalog/SDK/observability stack, and the Inspect-Design-Implement-Test-Validate-Document-Commit phase loop this whole build followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C146" s="11" t="inlineStr">
+        <is>
+          <t>AI Development Context: docs/architecture/overview.md kept current</t>
+        </is>
+      </c>
+      <c r="D146" s="11" t="inlineStr">
+        <is>
+          <t>Diagram and principles updated to include Keycloak/OpenFGA, the 3 SDKs, Backstage, the observability stack, and the Admin Portal - all previously entirely absent from the diagram</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>